<commit_message>
chore: Map legacy syllabus subjects to official RPSC subjects
- Mapped old generic subjects (like 'राजस्थान GK', 'विज्ञान', 'तर्कशक्ति') to the exact official RPSC Syllabus Subjects (e.g. 'राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत').
- Updated Firebase SYLLABUS_TOPICS collection to reflect this official mapping so that UI components like SyllabusTab and GapAnalysisTab render official subject names.
</commit_message>
<xml_diff>
--- a/Update_App_Data/ras_syllabus_data.xlsx
+++ b/Update_App_Data/ras_syllabus_data.xlsx
@@ -403,27 +403,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S183"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="40.83203125" customWidth="1"/>
-    <col min="14" max="14" width="50.83203125" customWidth="1"/>
-    <col min="15" max="15" width="35.83203125" customWidth="1"/>
-    <col min="16" max="16" width="14.83203125" customWidth="1"/>
-    <col min="17" max="17" width="30.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -492,7 +471,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C2" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D2" s="1" t="str">
         <v>—</v>
@@ -551,7 +530,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C3" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D3" s="1" t="str">
         <v>—</v>
@@ -610,7 +589,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C4" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D4" s="1" t="str">
         <v>—</v>
@@ -619,7 +598,7 @@
         <v>प्रमुख राजवंश एवं शासक (18वीं सदी तक)</v>
       </c>
       <c r="F4" s="1" t="str">
-        <v>मेवाड़ (बप्पा रावल, राणा कुम्भा, राणा सांगा, महाराणा प्रताप); मारवाड़; आमेर; बीकानेर; हाड़ौती</v>
+        <v>मेवाड़ (बप्पा रावल, राणा कुम्भा, राणा सांगा, महाराणा प्रताप), मारवाड़, आमेर, बीकानेर, हाड़ौती</v>
       </c>
       <c r="G4" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -669,7 +648,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C5" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D5" s="1" t="str">
         <v>—</v>
@@ -728,7 +707,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C6" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D6" s="1" t="str">
         <v>—</v>
@@ -787,7 +766,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C7" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D7" s="1" t="str">
         <v>—</v>
@@ -796,7 +775,7 @@
         <v>स्थापत्य कला: मंदिर, किले, महल, बावड़ियाँ</v>
       </c>
       <c r="F7" s="1" t="str">
-        <v>6 UNESCO किले (चित्तौड़, कुम्भलगढ़, रणथम्भौर, आमेर, जैसलमेर, गागरोन); दिलवाड़ा; चाँद बावड़ी</v>
+        <v>6 UNESCO किले (चित्तौड़, कुम्भलगढ़, रणथम्भौर, आमेर, जैसलमेर, गागरोन), दिलवाड़ा, चाँद बावड़ी</v>
       </c>
       <c r="G7" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -846,7 +825,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C8" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D8" s="1" t="str">
         <v>—</v>
@@ -855,7 +834,7 @@
         <v>चित्रकला स्कूल एवं हस्तशिल्प</v>
       </c>
       <c r="F8" s="1" t="str">
-        <v>मेवाड़, मारवाड़, किशनगढ़ (बणी-ठणी), बूँदी, कोटा स्कूल; नीली मिट्टी, ब्लू पॉटरी, बाँधनी</v>
+        <v>मेवाड़, मारवाड़, किशनगढ़ (बणी-ठणी), बूँदी, कोटा स्कूल, नीली मिट्टी, ब्लू पॉटरी, बाँधनी</v>
       </c>
       <c r="G8" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -905,7 +884,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C9" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D9" s="1" t="str">
         <v>—</v>
@@ -914,7 +893,7 @@
         <v>लोक नृत्य, संगीत एवं वाद्ययंत्र</v>
       </c>
       <c r="F9" s="1" t="str">
-        <v>घूमर, कालबेलिया (UNESCO 2010), गैर, तेरहताली, भवाई, चरी; मांड, लांगा; सारंगी, रावणहत्था</v>
+        <v>घूमर, कालबेलिया (UNESCO 2010), गैर, तेरहताली, भवाई, चरी, मांड, लांगा, सारंगी, रावणहत्था</v>
       </c>
       <c r="G9" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -964,7 +943,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C10" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D10" s="1" t="str">
         <v>—</v>
@@ -973,7 +952,7 @@
         <v>भाषा, साहित्य, संत एवं लोक देवता</v>
       </c>
       <c r="F10" s="1" t="str">
-        <v>डिंगल-पिंगल; पृथ्वीराज रासो; मीराबाई, रामदेवजी, तेजाजी, पाबूजी, गोगाजी, जाम्भोजी</v>
+        <v>डिंगल-पिंगल, पृथ्वीराज रासो, मीराबाई, रामदेवजी, तेजाजी, पाबूजी, गोगाजी, जाम्भोजी</v>
       </c>
       <c r="G10" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1023,7 +1002,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C11" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D11" s="1" t="str">
         <v>—</v>
@@ -1032,7 +1011,7 @@
         <v>मेले, त्यौहार, वेशभूषा एवं आभूषण</v>
       </c>
       <c r="F11" s="1" t="str">
-        <v>पुष्कर, नागौर, बेणेश्वर, रामदेवरा मेले; गणगौर, तीज; बोरला, हाँसली आभूषण</v>
+        <v>पुष्कर, नागौर, बेणेश्वर, रामदेवरा मेले, गणगौर, तीज, बोरला, हाँसली आभूषण</v>
       </c>
       <c r="G11" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1082,7 +1061,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C12" s="1" t="str">
-        <v>राजस्थान GK</v>
+        <v>राजस्थान का इतिहास, कला, संस्कृति, साहित्य, परम्परा एवं विरासत</v>
       </c>
       <c r="D12" s="1" t="str">
         <v>—</v>
@@ -1141,7 +1120,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C13" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D13" s="1" t="str">
         <v>प्राचीन</v>
@@ -1150,7 +1129,7 @@
         <v>सांस्कृतिक आधार: सिंधु एवं वैदिक युग; बौद्ध-जैन-आजीवक</v>
       </c>
       <c r="F13" s="1" t="str">
-        <v>सिंधु सभ्यता; वैदिक साहित्य (ऋग्वेद-उपनिषद); बौद्ध: 4 आर्य सत्य; जैन: त्रिरत्न</v>
+        <v>सिंधु सभ्यता, वैदिक साहित्य (ऋग्वेद-उपनिषद), बौद्ध: 4 आर्य सत्य, जैन: त्रिरत्न</v>
       </c>
       <c r="G13" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1200,7 +1179,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C14" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D14" s="1" t="str">
         <v>प्राचीन</v>
@@ -1209,7 +1188,7 @@
         <v>प्रमुख राजवंश: मौर्य, कुषाण, गुप्त, चालुक्य, पल्लव, चोल</v>
       </c>
       <c r="F14" s="1" t="str">
-        <v>अशोक (धम्म); समुद्रगुप्त 'भारत का नेपोलियन'; चंद्रगुप्त II; कनिष्क (गांधार कला); राजराज I</v>
+        <v>अशोक (धम्म), समुद्रगुप्त 'भारत का नेपोलियन', चंद्रगुप्त II, कनिष्क (गांधार कला), राजराज I</v>
       </c>
       <c r="G14" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1259,7 +1238,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C15" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D15" s="1" t="str">
         <v>प्राचीन</v>
@@ -1268,7 +1247,7 @@
         <v>कला, स्थापत्य एवं वैज्ञानिक विकास</v>
       </c>
       <c r="F15" s="1" t="str">
-        <v>साँची स्तूप, अजंता-एलोरा; आर्यभट्ट, ब्रह्मगुप्त; चरक-सुश्रुत</v>
+        <v>साँची स्तूप, अजंता-एलोरा, आर्यभट्ट, ब्रह्मगुप्त, चरक-सुश्रुत</v>
       </c>
       <c r="G15" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1318,7 +1297,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C16" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D16" s="1" t="str">
         <v>मध्यकाल</v>
@@ -1327,7 +1306,7 @@
         <v>सल्तनत काल एवं विजयनगर साम्राज्य</v>
       </c>
       <c r="F16" s="1" t="str">
-        <v>कुतुबुद्दीन ऐबक, अलाउद्दीन खिलजी, मुहम्मद-बिन-तुगलक; कृष्णदेवराय; हम्पी</v>
+        <v>कुतुबुद्दीन ऐबक, अलाउद्दीन खिलजी, मुहम्मद-बिन-तुगलक, कृष्णदेवराय, हम्पी</v>
       </c>
       <c r="G16" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1377,7 +1356,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C17" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D17" s="1" t="str">
         <v>मध्यकाल</v>
@@ -1386,7 +1365,7 @@
         <v>मुगल काल: प्रशासन, नीतियाँ एवं मराठा</v>
       </c>
       <c r="F17" s="1" t="str">
-        <v>अकबर (दीन-इलाही, नवरत्न, मनसबदारी); शाहजहाँ (ताजमहल); शिवाजी (अष्टप्रधान)</v>
+        <v>अकबर (दीन-इलाही, नवरत्न, मनसबदारी), शाहजहाँ (ताजमहल), शिवाजी (अष्टप्रधान)</v>
       </c>
       <c r="G17" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1436,7 +1415,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C18" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D18" s="1" t="str">
         <v>मध्यकाल</v>
@@ -1445,7 +1424,7 @@
         <v>धार्मिक आंदोलन: भक्ति एवं सूफी</v>
       </c>
       <c r="F18" s="1" t="str">
-        <v>कबीर, तुलसीदास, मीराबाई, सूरदास; ख्वाजा मोइनुद्दीन (चिश्ती-अजमेर); तानसेन</v>
+        <v>कबीर, तुलसीदास, मीराबाई, सूरदास, ख्वाजा मोइनुद्दीन (चिश्ती-अजमेर), तानसेन</v>
       </c>
       <c r="G18" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1495,7 +1474,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C19" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D19" s="1" t="str">
         <v>आधुनिक</v>
@@ -1504,7 +1483,7 @@
         <v>ब्रिटिश साम्राज्यवाद, 1857 का विद्रोह</v>
       </c>
       <c r="F19" s="1" t="str">
-        <v>एंग्लो-मैसूर (टीपू सुल्तान); 1857: मंगल पांडे, झाँसी की रानी, कुँवर सिंह; राजस्थान: नसीराबाद, आउवा</v>
+        <v>एंग्लो-मैसूर (टीपू सुल्तान), 1857: मंगल पांडे, झाँसी की रानी, कुँवर सिंह, राजस्थान: नसीराबाद, आउवा</v>
       </c>
       <c r="G19" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1554,7 +1533,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C20" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D20" s="1" t="str">
         <v>आधुनिक</v>
@@ -1563,7 +1542,7 @@
         <v>ब्रिटिश नीतियाँ; राष्ट्रवाद; सामाजिक-धार्मिक सुधार आंदोलन</v>
       </c>
       <c r="F20" s="1" t="str">
-        <v>स्थायी बंदोबस्त; INC 1885; ब्रह्म समाज (राममोहन राय); आर्य समाज (दयानंद); विवेकानंद</v>
+        <v>स्थायी बंदोबस्त, INC 1885, ब्रह्म समाज (राममोहन राय), आर्य समाज (दयानंद), विवेकानंद</v>
       </c>
       <c r="G20" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1613,7 +1592,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C21" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D21" s="1" t="str">
         <v>आधुनिक</v>
@@ -1622,7 +1601,7 @@
         <v>स्वतंत्रता संग्राम: विकास, चरण, प्रमुख घटनाएँ</v>
       </c>
       <c r="F21" s="1" t="str">
-        <v>असहयोग 1920, सविनय अवज्ञा 1930, भारत छोड़ो 1942; INA-Bose; भगत सिंह; विभाजन 1947</v>
+        <v>असहयोग 1920, सविनय अवज्ञा 1930, भारत छोड़ो 1942, INA-Bose, भगत सिंह, विभाजन 1947</v>
       </c>
       <c r="G21" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1672,7 +1651,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C22" s="1" t="str">
-        <v>भारत इतिहास</v>
+        <v>भारत का इतिहास</v>
       </c>
       <c r="D22" s="1" t="str">
         <v>आधुनिक</v>
@@ -1681,7 +1660,7 @@
         <v>स्वातंत्र्योत्तर राष्ट्र निर्माण (2000 तक)</v>
       </c>
       <c r="F22" s="1" t="str">
-        <v>SRC 1956; IIT-ISRO-DRDO स्थापना; हरित क्रांति; 1991 LPG सुधार</v>
+        <v>SRC 1956, IIT-ISRO-DRDO स्थापना, हरित क्रांति, 1991 LPG सुधार</v>
       </c>
       <c r="G22" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -1731,7 +1710,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C23" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D23" s="1" t="str">
         <v>—</v>
@@ -1790,7 +1769,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C24" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D24" s="1" t="str">
         <v>—</v>
@@ -1799,7 +1778,7 @@
         <v>विश्व की प्रमुख नदियाँ एवं झीलें</v>
       </c>
       <c r="F24" s="1" t="str">
-        <v>नील (longest), अमेजन (max water), बाइकाल (deepest); कैस्पियन (largest lake)</v>
+        <v>नील (longest), अमेजन (max water), बाइकाल (deepest), कैस्पियन (largest lake)</v>
       </c>
       <c r="G24" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1849,7 +1828,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C25" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D25" s="1" t="str">
         <v>—</v>
@@ -1858,7 +1837,7 @@
         <v>विश्व: प्राकृतिक वनस्पति एवं कृषि</v>
       </c>
       <c r="F25" s="1" t="str">
-        <v>Biomes: Tropical RF, Savanna, Prairies; गेहूँ-USA, चावल-SE Asia, कॉफी-Brazil</v>
+        <v>Biomes: Tropical RF, Savanna, Prairies, गेहूँ-USA, चावल-SE Asia, कॉफी-Brazil</v>
       </c>
       <c r="G25" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -1908,7 +1887,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C26" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D26" s="1" t="str">
         <v>—</v>
@@ -1917,7 +1896,7 @@
         <v>पर्यावरणीय मुद्दे: मरुस्थलीकरण, जलवायु परिवर्तन, ओजोन</v>
       </c>
       <c r="F26" s="1" t="str">
-        <v>Montreal Protocol 1987; Paris Agreement 2015; IPCC AR6; Carbon Credits; Amazon deforestation</v>
+        <v>Montreal Protocol 1987, Paris Agreement 2015, IPCC AR6, Carbon Credits, Amazon deforestation</v>
       </c>
       <c r="G26" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -1967,7 +1946,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C27" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D27" s="1" t="str">
         <v>—</v>
@@ -2026,7 +2005,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C28" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D28" s="1" t="str">
         <v>—</v>
@@ -2035,7 +2014,7 @@
         <v>भारत की जलवायु एवं मानसून</v>
       </c>
       <c r="F28" s="1" t="str">
-        <v>ITCZ, SW मानसून (जून-Sept), NE मानसून (TN); El Nino/La Nina; चेरापूँजी</v>
+        <v>ITCZ, SW मानसून (जून-Sept), NE मानसून (TN), El Nino/La Nina, चेरापूँजी</v>
       </c>
       <c r="G28" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2085,7 +2064,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C29" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D29" s="1" t="str">
         <v>—</v>
@@ -2094,7 +2073,7 @@
         <v>भारत: प्रमुख नदियाँ, झीलें एवं सिंचाई</v>
       </c>
       <c r="F29" s="1" t="str">
-        <v>गंगा, ब्रह्मपुत्र, नर्मदा (पश्चिम बहाव), कावेरी; चिल्का, वुलर, लोकटक; टेहरी, भाखड़ा</v>
+        <v>गंगा, ब्रह्मपुत्र, नर्मदा (पश्चिम बहाव), कावेरी, चिल्का, वुलर, लोकटक, टेहरी, भाखड़ा</v>
       </c>
       <c r="G29" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2144,7 +2123,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C30" s="1" t="str">
-        <v>भूगोल</v>
+        <v>विश्व एवं भारत का भूगोल</v>
       </c>
       <c r="D30" s="1" t="str">
         <v>—</v>
@@ -2153,7 +2132,7 @@
         <v>भारत: फसलें एवं खनिज</v>
       </c>
       <c r="F30" s="1" t="str">
-        <v>खरीफ-रबी-जायद; लौह (Jharkhand), बॉक्साइट (Odisha), कोयला (Jharkhand), पेट्रो (Mumbai High)</v>
+        <v>खरीफ-रबी-जायद, लौह (Jharkhand), बॉक्साइट (Odisha), कोयला (Jharkhand), पेट्रो (Mumbai High)</v>
       </c>
       <c r="G30" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2203,7 +2182,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C31" s="1" t="str">
-        <v>भूगोल</v>
+        <v>राजस्थान का भूगोल</v>
       </c>
       <c r="D31" s="1" t="str">
         <v>—</v>
@@ -2212,7 +2191,7 @@
         <v>राजस्थान का भौतिक विभाजन</v>
       </c>
       <c r="F31" s="1" t="str">
-        <v>4 भाग: पश्चिमी मरुस्थल 61%, अरावली, पूर्वी मैदान, दक्षिण-पूर्वी पठार; क्षेत्रफल 3,42,239 km²</v>
+        <v>4 भाग: पश्चिमी मरुस्थल 61%, अरावली, पूर्वी मैदान, दक्षिण-पूर्वी पठार, क्षेत्रफल 3, 42, 239 km²</v>
       </c>
       <c r="G31" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2262,7 +2241,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C32" s="1" t="str">
-        <v>भूगोल</v>
+        <v>राजस्थान का भूगोल</v>
       </c>
       <c r="D32" s="1" t="str">
         <v>—</v>
@@ -2271,7 +2250,7 @@
         <v>राजस्थान की नदियाँ एवं झीलें</v>
       </c>
       <c r="F32" s="1" t="str">
-        <v>लूणी (अरब सागर), चम्बल-बनास (बंगाल), घग्गर (मृत); सांभर (खारी), पिचोला, राजसमंद</v>
+        <v>लूणी (अरब सागर), चम्बल-बनास (बंगाल), घग्गर (मृत), सांभर (खारी), पिचोला, राजसमंद</v>
       </c>
       <c r="G32" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2321,7 +2300,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C33" s="1" t="str">
-        <v>भूगोल</v>
+        <v>राजस्थान का भूगोल</v>
       </c>
       <c r="D33" s="1" t="str">
         <v>—</v>
@@ -2330,7 +2309,7 @@
         <v>राजस्थान: जलवायु, वनस्पति, जैव विविधता</v>
       </c>
       <c r="F33" s="1" t="str">
-        <v>Koppen BWhw/BShs/Caw; लू; गोडावण (State Bird); रणथम्भौर, सरिस्का, केवलादेव (UNESCO WH)</v>
+        <v>Koppen BWhw/BShs/Caw, लू, गोडावण (State Bird), रणथम्भौर, सरिस्का, केवलादेव (UNESCO WH)</v>
       </c>
       <c r="G33" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2380,7 +2359,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C34" s="1" t="str">
-        <v>भूगोल</v>
+        <v>राजस्थान का भूगोल</v>
       </c>
       <c r="D34" s="1" t="str">
         <v>—</v>
@@ -2389,7 +2368,7 @@
         <v>राजस्थान: मृदा, कृषि, पशुधन, सिंचाई</v>
       </c>
       <c r="F34" s="1" t="str">
-        <v>रेतीली, जलोढ़, काली; बाजरा-सरसों-1st; ऊँट, भेड़; IGNP (Beas-Sutlej); ड्रिप सिंचाई</v>
+        <v>रेतीली, जलोढ़, काली, बाजरा-सरसों-1st, ऊँट, भेड़, IGNP (Beas-Sutlej), ड्रिप सिंचाई</v>
       </c>
       <c r="G34" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2439,7 +2418,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C35" s="1" t="str">
-        <v>भूगोल</v>
+        <v>राजस्थान का भूगोल</v>
       </c>
       <c r="D35" s="1" t="str">
         <v>—</v>
@@ -2448,7 +2427,7 @@
         <v>राजस्थान: जनसंख्या, जनजातियाँ, खनिज, पर्यटन</v>
       </c>
       <c r="F35" s="1" t="str">
-        <v>6.86 cr (2011); साक्षरता 66.1%; भील (max ST); जस्ता-जावर, संगमरमर-मकराना, तांबा-खेतड़ी</v>
+        <v>6.86 cr (2011), साक्षरता 66.1%, भील (max ST), जस्ता-जावर, संगमरमर-मकराना, तांबा-खेतड़ी</v>
       </c>
       <c r="G35" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2498,7 +2477,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C36" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>भारतीय संविधान, राजनीतिक व्यवस्था और शासन</v>
       </c>
       <c r="D36" s="1" t="str">
         <v>—</v>
@@ -2507,7 +2486,7 @@
         <v>संविधान निर्माण, उद्देशिका, नागरिकता, FR, DPSP, FD</v>
       </c>
       <c r="F36" s="1" t="str">
-        <v>Constituent Assembly; उद्देशिका (42वाँ संशोधन 1976); FR: अनु.12-35; DPSP: 36-51; FD: 51-A</v>
+        <v>Constituent Assembly, उद्देशिका (42वाँ संशोधन 1976), FR: अनु.12-35, DPSP: 36-51, FD: 51-A</v>
       </c>
       <c r="G36" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2557,7 +2536,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C37" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>भारतीय संविधान, राजनीतिक व्यवस्था और शासन</v>
       </c>
       <c r="D37" s="1" t="str">
         <v>—</v>
@@ -2566,7 +2545,7 @@
         <v>संघीय सरकार: कार्यपालिका, विधायिका, न्यायपालिका</v>
       </c>
       <c r="F37" s="1" t="str">
-        <v>राष्ट्रपति: अनु.52-62, Emergency powers; PM+Cabinet; Lok Sabha 543, RS 250; SC: PIL, Judicial Review</v>
+        <v>राष्ट्रपति: अनु.52-62, Emergency powers, PM+Cabinet, Lok Sabha 543, RS 250, SC: PIL, Judicial Review</v>
       </c>
       <c r="G37" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2616,7 +2595,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C38" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>भारतीय संविधान, राजनीतिक व्यवस्था और शासन</v>
       </c>
       <c r="D38" s="1" t="str">
         <v>—</v>
@@ -2625,7 +2604,7 @@
         <v>संघ-राज्य संबंध; आपातकालीन प्रावधान</v>
       </c>
       <c r="F38" s="1" t="str">
-        <v>7वीं अनुसूची: 3 Lists; अनु.356 President Rule; अनु.352 National Emergency; अनु.360 Financial Emergency</v>
+        <v>7वीं अनुसूची: 3 Lists, अनु.356 President Rule, अनु.352 National Emergency, अनु.360 Financial Emergency</v>
       </c>
       <c r="G38" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2675,7 +2654,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C39" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>भारतीय संविधान, राजनीतिक व्यवस्था और शासन</v>
       </c>
       <c r="D39" s="1" t="str">
         <v>—</v>
@@ -2684,7 +2663,7 @@
         <v>स्थानीय सरकार: पंचायती राज एवं नगरपालिकाएँ</v>
       </c>
       <c r="F39" s="1" t="str">
-        <v>73वाँ संशोधन 1992 (Panchayati Raj 3-tier); 74वाँ (ULBs); PESA Act 1996 (Tribal areas)</v>
+        <v>73वाँ संशोधन 1992 (Panchayati Raj 3-tier), 74वाँ (ULBs), PESA Act 1996 (Tribal areas)</v>
       </c>
       <c r="G39" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2734,7 +2713,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C40" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>भारतीय संविधान, राजनीतिक व्यवस्था और शासन</v>
       </c>
       <c r="D40" s="1" t="str">
         <v>—</v>
@@ -2743,7 +2722,7 @@
         <v>निर्वाचन आयोग, UPSC, NHRC, NCPCR, NCWC, NITI Aayog</v>
       </c>
       <c r="F40" s="1" t="str">
-        <v>ECI: अनु.324; UPSC: 315-323; NHRC: HR Protection Act 1993; NITI Aayog: 2015 (replaced PC); CAG: 148</v>
+        <v>ECI: अनु.324, UPSC: 315-323, NHRC: HR Protection Act 1993, NITI Aayog: 2015 (replaced PC), CAG: 148</v>
       </c>
       <c r="G40" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2793,7 +2772,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C41" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>भारतीय संविधान, राजनीतिक व्यवस्था और शासन</v>
       </c>
       <c r="D41" s="1" t="str">
         <v>—</v>
@@ -2802,7 +2781,7 @@
         <v>लोक नीति, RTI, Lokpal, CVC, CIC</v>
       </c>
       <c r="F41" s="1" t="str">
-        <v>RTI Act 2005 (Sec.8 exemptions); Lokpal Act 2013; CVC: 1964, Santhanam Committee; CPGRAMS grievance</v>
+        <v>RTI Act 2005 (Sec.8 exemptions), Lokpal Act 2013, CVC: 1964, Santhanam Committee, CPGRAMS grievance</v>
       </c>
       <c r="G41" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2852,7 +2831,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C42" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>राजस्थान की राजनीतिक एवं प्रशासनिक व्यवस्था</v>
       </c>
       <c r="D42" s="1" t="str">
         <v>—</v>
@@ -2861,7 +2840,7 @@
         <v>राजस्थान: राज्यपाल, CM, विधानसभा, HC, AG</v>
       </c>
       <c r="F42" s="1" t="str">
-        <v>राज्यपाल: discretionary powers; विधानसभा 200 seats; HC: Jodhpur + Jaipur bench; AG: अनु.165</v>
+        <v>राज्यपाल: discretionary powers, विधानसभा 200 seats, HC: Jodhpur + Jaipur bench, AG: अनु.165</v>
       </c>
       <c r="G42" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2911,7 +2890,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C43" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>राजस्थान की राजनीतिक एवं प्रशासनिक व्यवस्था</v>
       </c>
       <c r="D43" s="1" t="str">
         <v>—</v>
@@ -2920,7 +2899,7 @@
         <v>राजस्थान: मुख्य सचिव, Collector, SP, SDO, तहसीलदार</v>
       </c>
       <c r="F43" s="1" t="str">
-        <v>Admin hierarchy: Chief Secretary → Commissioner → Collector → SDM → Tehsildar; 7 Divisions</v>
+        <v>Admin hierarchy: Chief Secretary → Commissioner → Collector → SDM → Tehsildar, 7 Divisions</v>
       </c>
       <c r="G43" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -2970,7 +2949,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C44" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>राजस्थान की राजनीतिक एवं प्रशासनिक व्यवस्था</v>
       </c>
       <c r="D44" s="1" t="str">
         <v>—</v>
@@ -2979,7 +2958,7 @@
         <v>RPSC, RSEC, RSIC, Revenue Board, Lokayukta</v>
       </c>
       <c r="F44" s="1" t="str">
-        <v>RPSC: Art.315; RSEC: SEA; RSIC: RTI Act; Revenue Board: Ajmer; Lokayukta: Raj Act 1973</v>
+        <v>RPSC: Art.315, RSEC: SEA, RSIC: RTI Act, Revenue Board: Ajmer, Lokayukta: Raj Act 1973</v>
       </c>
       <c r="G44" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3029,7 +3008,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C45" s="1" t="str">
-        <v>राज्यव्यवस्था</v>
+        <v>राजस्थान की राजनीतिक एवं प्रशासनिक व्यवस्था</v>
       </c>
       <c r="D45" s="1" t="str">
         <v>—</v>
@@ -3038,7 +3017,7 @@
         <v>राजस्थान: पंचायती राज एवं नगरपालिका प्रशासन</v>
       </c>
       <c r="F45" s="1" t="str">
-        <v>Raj. PR Act 1994; 3-tier: GP(Sarpanch), PS(Pradhan), ZP(Zila Pramukh); 7 Nagar Nigam in Raj.</v>
+        <v>Raj. PR Act 1994, 3-tier: GP(Sarpanch), PS(Pradhan), ZP(Zila Pramukh), 7 Nagar Nigam in Raj.</v>
       </c>
       <c r="G45" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3088,7 +3067,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C46" s="1" t="str">
-        <v>अर्थव्यवस्था</v>
+        <v>आर्थिक अवधारणाएँ एवं भारतीय अर्थव्यवस्था</v>
       </c>
       <c r="D46" s="1" t="str">
         <v>—</v>
@@ -3097,7 +3076,7 @@
         <v>आर्थिक संवृद्धि, विकास एवं सतत विकास; HDI, SDG</v>
       </c>
       <c r="F46" s="1" t="str">
-        <v>GDP/GNP/NNP; HDI (UNDP 4 components); SDG 17 goals; Green GDP; Inclusive Growth; India HDI rank</v>
+        <v>GDP/GNP/NNP, HDI (UNDP 4 components), SDG 17 goals, Green GDP, Inclusive Growth, India HDI rank</v>
       </c>
       <c r="G46" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3147,7 +3126,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C47" s="1" t="str">
-        <v>अर्थव्यवस्था</v>
+        <v>आर्थिक अवधारणाएँ एवं भारतीय अर्थव्यवस्था</v>
       </c>
       <c r="D47" s="1" t="str">
         <v>—</v>
@@ -3156,7 +3135,7 @@
         <v>मौद्रिक एवं राजकोषीय नीति; नवीनतम बजट; GST</v>
       </c>
       <c r="F47" s="1" t="str">
-        <v>Repo Rate, CRR, SLR; FRBM Act 2003; Fiscal Deficit; Union Budget 2025-26 highlights; GST slabs 0/5/12/18/28%</v>
+        <v>Repo Rate, CRR, SLR, FRBM Act 2003, Fiscal Deficit, Union Budget 2025-26 highlights, GST slabs 0/5/12/18/28%</v>
       </c>
       <c r="G47" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3206,7 +3185,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C48" s="1" t="str">
-        <v>अर्थव्यवस्था</v>
+        <v>आर्थिक अवधारणाएँ एवं भारतीय अर्थव्यवस्था</v>
       </c>
       <c r="D48" s="1" t="str">
         <v>—</v>
@@ -3215,7 +3194,7 @@
         <v>राजकोषीय संघवाद; वित्त आयोग; कृषि विकास</v>
       </c>
       <c r="F48" s="1" t="str">
-        <v>15th FC (NK Singh): 41% devolution; Art.280; MSP-CACP; PM-KISAN; e-NAM; FPO; Land reforms</v>
+        <v>15th FC (NK Singh): 41% devolution, Art.280, MSP-CACP, PM-KISAN, e-NAM, FPO, Land reforms</v>
       </c>
       <c r="G48" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3265,7 +3244,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C49" s="1" t="str">
-        <v>अर्थव्यवस्था</v>
+        <v>आर्थिक अवधारणाएँ एवं भारतीय अर्थव्यवस्था</v>
       </c>
       <c r="D49" s="1" t="str">
         <v>—</v>
@@ -3274,7 +3253,7 @@
         <v>औद्योगिक नीति: LPG 1991; MSME; Make in India</v>
       </c>
       <c r="F49" s="1" t="str">
-        <v>New Industrial Policy 1991 (Dr Manmohan Singh); MSME definition (2020); PLI; Start-up India; FDI vs FII</v>
+        <v>New Industrial Policy 1991 (Dr Manmohan Singh), MSME definition (2020), PLI, Start-up India, FDI vs FII</v>
       </c>
       <c r="G49" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3324,7 +3303,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C50" s="1" t="str">
-        <v>अर्थव्यवस्था</v>
+        <v>आर्थिक अवधारणाएँ एवं भारतीय अर्थव्यवस्था</v>
       </c>
       <c r="D50" s="1" t="str">
         <v>—</v>
@@ -3333,7 +3312,7 @@
         <v>सामाजिक न्याय: MGNREGA, PM Jan Dhan, Ayushman Bharat</v>
       </c>
       <c r="F50" s="1" t="str">
-        <v>MGNREGA: 100 days, Job card, Schedule I wage; PM Jan Dhan: zero balance; Ayushman Bharat: ₹5 lakh cover</v>
+        <v>MGNREGA: 100 days, Job card, Schedule I wage, PM Jan Dhan: zero balance, Ayushman Bharat: ₹5 lakh cover</v>
       </c>
       <c r="G50" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3383,7 +3362,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C51" s="1" t="str">
-        <v>अर्थव्यवस्था</v>
+        <v>राजस्थान की अर्थव्यवस्था</v>
       </c>
       <c r="D51" s="1" t="str">
         <v>—</v>
@@ -3392,7 +3371,7 @@
         <v>राजस्थान अर्थव्यवस्था: GSDP, कृषि-उद्योग-सेवा</v>
       </c>
       <c r="F51" s="1" t="str">
-        <v>GSDP ~₹14 lakh cr; Agriculture: बाजरा-सरसों-जीरा 1st in India; Zinc (Vedanta-HZL); Bhadla Solar Park</v>
+        <v>GSDP ~₹14 lakh cr, Agriculture: बाजरा-सरसों-जीरा 1st in India, Zinc (Vedanta-HZL), Bhadla Solar Park</v>
       </c>
       <c r="G51" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3442,7 +3421,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C52" s="1" t="str">
-        <v>अर्थव्यवस्था</v>
+        <v>राजस्थान की अर्थव्यवस्था</v>
       </c>
       <c r="D52" s="1" t="str">
         <v>—</v>
@@ -3451,7 +3430,7 @@
         <v>राजस्थान: ऊर्जा एवं सरकारी योजनाएँ</v>
       </c>
       <c r="F52" s="1" t="str">
-        <v>Solar capacity 1st in India (~20,000 MW); Chiranjeevi Health Insurance; Indira Rasoi (₹8/plate); Jan Aadhaar</v>
+        <v>Solar capacity 1st in India (~20, 000 MW), Chiranjeevi Health Insurance, Indira Rasoi (₹8/plate), Jan Aadhaar</v>
       </c>
       <c r="G52" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3501,7 +3480,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C53" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D53" s="1" t="str">
         <v>—</v>
@@ -3560,7 +3539,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C54" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D54" s="1" t="str">
         <v>—</v>
@@ -3619,7 +3598,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C55" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D55" s="1" t="str">
         <v>—</v>
@@ -3628,7 +3607,7 @@
         <v>जीव विज्ञान: कोशिका, रक्त समूह, मेंडल के नियम</v>
       </c>
       <c r="F55" s="1" t="str">
-        <v>कोशिका: Prokaryote-Eukaryote; रक्त: ABO+Rh (O- universal donor, AB+ universal recipient); मेंडल</v>
+        <v>कोशिका: Prokaryote-Eukaryote, रक्त: ABO+Rh (O- universal donor, AB+ universal recipient), मेंडल</v>
       </c>
       <c r="G55" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3678,7 +3657,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C56" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D56" s="1" t="str">
         <v>—</v>
@@ -3687,7 +3666,7 @@
         <v>ICT: कम्प्यूटर, इंटरनेट, AI, Cyber Security</v>
       </c>
       <c r="F56" s="1" t="str">
-        <v>RAM vs ROM; Input-Output; OS; AI/ML/DL basics; Blockchain; IoT; 5G; Cyber threats: Phishing, Malware, 2FA</v>
+        <v>RAM vs ROM, Input-Output, OS, AI/ML/DL basics, Blockchain, IoT, 5G, Cyber threats: Phishing, Malware, 2FA</v>
       </c>
       <c r="G56" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3737,7 +3716,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C57" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D57" s="1" t="str">
         <v>—</v>
@@ -3746,7 +3725,7 @@
         <v>अंतरिक्ष एवं रक्षा प्रौद्योगिकी</v>
       </c>
       <c r="F57" s="1" t="str">
-        <v>Chandrayaan-3 (Aug 2023, Shiv Shakti Point), Aditya-L1, PSLV/LVM3; Agni-V (MIRV), BrahMos; HAL Tejas</v>
+        <v>Chandrayaan-3 (Aug 2023, Shiv Shakti Point), Aditya-L1, PSLV/LVM3, Agni-V (MIRV), BrahMos, HAL Tejas</v>
       </c>
       <c r="G57" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3796,7 +3775,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C58" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D58" s="1" t="str">
         <v>—</v>
@@ -3805,7 +3784,7 @@
         <v>जैव-प्रौद्योगिकी एवं नैनो-प्रौद्योगिकी</v>
       </c>
       <c r="F58" s="1" t="str">
-        <v>GMO: Bt Cotton (Cry gene); CRISPR-Cas9 (Nobel 2020); mRNA vaccine (COVID); Quantum Computing</v>
+        <v>GMO: Bt Cotton (Cry gene), CRISPR-Cas9 (Nobel 2020), mRNA vaccine (COVID), Quantum Computing</v>
       </c>
       <c r="G58" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3855,7 +3834,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C59" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D59" s="1" t="str">
         <v>—</v>
@@ -3864,7 +3843,7 @@
         <v>मानव स्वास्थ्य: रोग, पोषण, सार्वजनिक स्वास्थ्य</v>
       </c>
       <c r="F59" s="1" t="str">
-        <v>Malaria (Plasmodium-Anopheles), TB (Mycobacterium), Dengue (Aedes); Vitamins deficiency diseases</v>
+        <v>Malaria (Plasmodium-Anopheles), TB (Mycobacterium), Dengue (Aedes), Vitamins deficiency diseases</v>
       </c>
       <c r="G59" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3914,7 +3893,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C60" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D60" s="1" t="str">
         <v>—</v>
@@ -3923,7 +3902,7 @@
         <v>पर्यावरण एवं जैव विविधता</v>
       </c>
       <c r="F60" s="1" t="str">
-        <v>Ecosystem food chain-web; Biodiversity hotspots (India 4); IUCN categories; Paris Agreement; CBD 1992</v>
+        <v>Ecosystem food chain-web, Biodiversity hotspots (India 4), IUCN categories, Paris Agreement, CBD 1992</v>
       </c>
       <c r="G60" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -3973,7 +3952,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C61" s="1" t="str">
-        <v>विज्ञान</v>
+        <v>विज्ञान एवं प्रौद्योगिकी</v>
       </c>
       <c r="D61" s="1" t="str">
         <v>—</v>
@@ -3982,7 +3961,7 @@
         <v>राजस्थान S&amp;T; भारतीय वैज्ञानिकों का योगदान</v>
       </c>
       <c r="F61" s="1" t="str">
-        <v>CAZRI (Jodhpur); MPUAT (Udaipur); RAJUVAS (Bikaner); CV Raman, APJ Kalam, Homi Bhabha; Digital India</v>
+        <v>CAZRI (Jodhpur), MPUAT (Udaipur), RAJUVAS (Bikaner), CV Raman, APJ Kalam, Homi Bhabha, Digital India</v>
       </c>
       <c r="G61" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4032,7 +4011,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C62" s="1" t="str">
-        <v>तर्कशक्ति</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D62" s="1" t="str">
         <v>—</v>
@@ -4041,7 +4020,7 @@
         <v>कथन एवं मान्यताएँ</v>
       </c>
       <c r="F62" s="1" t="str">
-        <v>Implicit/Explicit assumption; Syllogism; 'सभी/कुछ/कोई नहीं' pattern</v>
+        <v>Implicit/Explicit assumption, Syllogism, 'सभी/कुछ/कोई नहीं' pattern</v>
       </c>
       <c r="G62" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4091,7 +4070,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C63" s="1" t="str">
-        <v>तर्कशक्ति</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D63" s="1" t="str">
         <v>—</v>
@@ -4100,7 +4079,7 @@
         <v>कथन एवं तर्क</v>
       </c>
       <c r="F63" s="1" t="str">
-        <v>Strong vs Weak argument; Cause-Effect; Analogy; Critical Reasoning</v>
+        <v>Strong vs Weak argument, Cause-Effect, Analogy, Critical Reasoning</v>
       </c>
       <c r="G63" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4150,7 +4129,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C64" s="1" t="str">
-        <v>तर्कशक्ति</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D64" s="1" t="str">
         <v>—</v>
@@ -4159,7 +4138,7 @@
         <v>कथन एवं निष्कर्ष / कार्यवाही</v>
       </c>
       <c r="F64" s="1" t="str">
-        <v>Definitely/Possibly follows; Practical course of action</v>
+        <v>Definitely/Possibly follows, Practical course of action</v>
       </c>
       <c r="G64" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4209,7 +4188,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C65" s="1" t="str">
-        <v>तर्कशक्ति</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D65" s="1" t="str">
         <v>—</v>
@@ -4218,7 +4197,7 @@
         <v>विश्लेषणात्मक तर्क: रैंकिंग, बैठक, दिशा ज्ञान, सम्बन्ध</v>
       </c>
       <c r="F65" s="1" t="str">
-        <v>Seating (circular+linear); Blood relations (family tree); Direction test; Venn diagram</v>
+        <v>Seating (circular+linear), Blood relations (family tree), Direction test, Venn diagram</v>
       </c>
       <c r="G65" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4268,7 +4247,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C66" s="1" t="str">
-        <v>तर्कशक्ति</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D66" s="1" t="str">
         <v>—</v>
@@ -4277,7 +4256,7 @@
         <v>संख्या/अक्षर अनुक्रम</v>
       </c>
       <c r="F66" s="1" t="str">
-        <v>Arithmetic, Prime, Fibonacci, Mixed series; Alphabet: EJOTY pattern; Position-based</v>
+        <v>Arithmetic, Prime, Fibonacci, Mixed series, Alphabet: EJOTY pattern, Position-based</v>
       </c>
       <c r="G66" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4327,7 +4306,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C67" s="1" t="str">
-        <v>तर्कशक्ति</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D67" s="1" t="str">
         <v>—</v>
@@ -4386,7 +4365,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C68" s="1" t="str">
-        <v>तर्कशक्ति</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D68" s="1" t="str">
         <v>—</v>
@@ -4395,7 +4374,7 @@
         <v>तार्किक वेन आरेख एवं आकार विभाजन</v>
       </c>
       <c r="F68" s="1" t="str">
-        <v>2-circle, 3-circle Venn; Count triangles-squares; Paper folding; Water-Mirror images</v>
+        <v>2-circle, 3-circle Venn, Count triangles-squares, Paper folding, Water-Mirror images</v>
       </c>
       <c r="G68" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4445,7 +4424,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C69" s="1" t="str">
-        <v>गणित</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D69" s="1" t="str">
         <v>—</v>
@@ -4454,7 +4433,7 @@
         <v>अनुपात-समानुपात, साझा, लाभ-हानि</v>
       </c>
       <c r="F69" s="1" t="str">
-        <v>Ratio a:b; Partnership = Capital×Time; CP-SP-Profit%; Discount; Marked Price</v>
+        <v>Ratio a:b, Partnership = Capital×Time, CP-SP-Profit%, Discount, Marked Price</v>
       </c>
       <c r="G69" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4504,7 +4483,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C70" s="1" t="str">
-        <v>गणित</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D70" s="1" t="str">
         <v>—</v>
@@ -4513,7 +4492,7 @@
         <v>प्रतिशत, सामान्य एवं चक्रवृद्धि ब्याज</v>
       </c>
       <c r="F70" s="1" t="str">
-        <v>% change; SI=PRT/100; CI=P(1+R/100)^T; CI-SI difference (2yr: PR²/10000)</v>
+        <v>% change, SI=PRT/100, CI=P(1+R/100)^T, CI-SI difference (2yr: PR²/10000)</v>
       </c>
       <c r="G70" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4563,7 +4542,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C71" s="1" t="str">
-        <v>गणित</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D71" s="1" t="str">
         <v>—</v>
@@ -4622,7 +4601,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C72" s="1" t="str">
-        <v>गणित</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D72" s="1" t="str">
         <v>—</v>
@@ -4681,7 +4660,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C73" s="1" t="str">
-        <v>गणित</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D73" s="1" t="str">
         <v>—</v>
@@ -4690,7 +4669,7 @@
         <v>माध्य, माध्यिका, बहुलक</v>
       </c>
       <c r="F73" s="1" t="str">
-        <v>AM=ΣX/n; GM=(x₁×...×xₙ)^1/n; HM=n/(Σ1/x); Median-Mode; AM≥GM≥HM</v>
+        <v>AM=ΣX/n, GM=(x₁×...×xₙ)^1/n, HM=n/(Σ1/x), Median-Mode, AM≥GM≥HM</v>
       </c>
       <c r="G73" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4740,7 +4719,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C74" s="1" t="str">
-        <v>गणित</v>
+        <v>तार्किक विवेचन एवं मानसिक योग्यता</v>
       </c>
       <c r="D74" s="1" t="str">
         <v>—</v>
@@ -4749,7 +4728,7 @@
         <v>क्रमचय, संचय एवं प्रायिकता</v>
       </c>
       <c r="F74" s="1" t="str">
-        <v>nPr=n!/(n-r)!; nCr=n!/r!(n-r)!; P=Favourable/Total; Dice-Card-Coin problems</v>
+        <v>nPr=n!/(n-r)!, nCr=n!/r!(n-r)!, P=Favourable/Total, Dice-Card-Coin problems</v>
       </c>
       <c r="G74" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4799,7 +4778,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C75" s="1" t="str">
-        <v>समसामयिक</v>
+        <v>समसामयिक घटनाएँ एवं मुद्दे (राजस्थान के विशेष संदर्भ में)</v>
       </c>
       <c r="D75" s="1" t="str">
         <v>—</v>
@@ -4808,7 +4787,7 @@
         <v>महत्वपूर्ण व्यक्तित्व एवं नियुक्तियाँ</v>
       </c>
       <c r="F75" s="1" t="str">
-        <v>CJI, RBI Governor, Election Commissioner, CAG; Noble Prize 2024-25; Bharat Ratna 2024</v>
+        <v>CJI, RBI Governor, Election Commissioner, CAG, Noble Prize 2024-25, Bharat Ratna 2024</v>
       </c>
       <c r="G75" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4858,7 +4837,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C76" s="1" t="str">
-        <v>समसामयिक</v>
+        <v>समसामयिक घटनाएँ एवं मुद्दे (राजस्थान के विशेष संदर्भ में)</v>
       </c>
       <c r="D76" s="1" t="str">
         <v>—</v>
@@ -4867,7 +4846,7 @@
         <v>नई योजनाएँ, कार्यक्रम एवं पहल</v>
       </c>
       <c r="F76" s="1" t="str">
-        <v>PM Internship Scheme; Viksit Bharat 2047; Rajasthan Investment Summit; Lakhpati Didi</v>
+        <v>PM Internship Scheme, Viksit Bharat 2047, Rajasthan Investment Summit, Lakhpati Didi</v>
       </c>
       <c r="G76" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4917,7 +4896,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C77" s="1" t="str">
-        <v>समसामयिक</v>
+        <v>समसामयिक घटनाएँ एवं मुद्दे (राजस्थान के विशेष संदर्भ में)</v>
       </c>
       <c r="D77" s="1" t="str">
         <v>—</v>
@@ -4926,7 +4905,7 @@
         <v>प्रमुख आर्थिक एवं राजनीतिक घटनाक्रम</v>
       </c>
       <c r="F77" s="1" t="str">
-        <v>India GDP 2024-25; G20 New Delhi 2023; BRICS expansion; Rajasthan 2023 elections</v>
+        <v>India GDP 2024-25, G20 New Delhi 2023, BRICS expansion, Rajasthan 2023 elections</v>
       </c>
       <c r="G77" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -4976,7 +4955,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C78" s="1" t="str">
-        <v>समसामयिक</v>
+        <v>समसामयिक घटनाएँ एवं मुद्दे (राजस्थान के विशेष संदर्भ में)</v>
       </c>
       <c r="D78" s="1" t="str">
         <v>—</v>
@@ -4985,7 +4964,7 @@
         <v>खेल एवं पुरस्कार</v>
       </c>
       <c r="F78" s="1" t="str">
-        <v>Olympics Paris 2024 (Neeraj-Silver, Manu Bhaker-2Bronze); ICC T20 WC 2024 India; Chess: Gukesh</v>
+        <v>Olympics Paris 2024 (Neeraj-Silver, Manu Bhaker-2Bronze), ICC T20 WC 2024 India, Chess: Gukesh</v>
       </c>
       <c r="G78" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5035,7 +5014,7 @@
         <v>Prelims GS1</v>
       </c>
       <c r="C79" s="1" t="str">
-        <v>समसामयिक</v>
+        <v>समसामयिक घटनाएँ एवं मुद्दे (राजस्थान के विशेष संदर्भ में)</v>
       </c>
       <c r="D79" s="1" t="str">
         <v>—</v>
@@ -5044,7 +5023,7 @@
         <v>राजस्थान सार्वजनिक परीक्षा (अनुचित साधन) अधिनियम 2022</v>
       </c>
       <c r="F79" s="1" t="str">
-        <v>Key provisions: 3 yr jail+₹10L; प्रश्नपत्र लीक: 10 yr+₹10 cr; 2 yr exam ban on conviction</v>
+        <v>Key provisions: 3 yr jail+₹10L, प्रश्नपत्र लीक: 10 yr+₹10 cr, 2 yr exam ban on conviction</v>
       </c>
       <c r="G79" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5103,7 +5082,7 @@
         <v>प्रागैतिहासिक संस्कृति एवं पुरातात्त्विक स्थल</v>
       </c>
       <c r="F80" s="1" t="str">
-        <v>Kalibangan IVC; Ahar Chalcolithic; Ganeshwar copper; Balathal; Bairath Mauryan</v>
+        <v>Kalibangan IVC, Ahar Chalcolithic, Ganeshwar copper, Balathal, Bairath Mauryan</v>
       </c>
       <c r="G80" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5162,7 +5141,7 @@
         <v>राजस्व एवं प्रशासनिक व्यवस्था (बदलते स्वरूप)</v>
       </c>
       <c r="F81" s="1" t="str">
-        <v>Jagirdari; Mansabdari; Batai/Kankut; Khalsa; Tarf-Pargana; Basta system</v>
+        <v>Jagirdari, Mansabdari, Batai/Kankut, Khalsa, Tarf-Pargana, Basta system</v>
       </c>
       <c r="G81" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5221,7 +5200,7 @@
         <v>19-20वीं सदी: किसान, आदिवासी, प्रजामंडल, एकीकरण</v>
       </c>
       <c r="F82" s="1" t="str">
-        <v>Bijolia (Vijay Singh Pathik); Bhil (Motilal Tejawat); Mewar PM (Maniklal Verma); 7 stages integration</v>
+        <v>Bijolia (Vijay Singh Pathik), Bhil (Motilal Tejawat), Mewar PM (Maniklal Verma), 7 stages integration</v>
       </c>
       <c r="G82" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5280,7 +5259,7 @@
         <v>राजस्थान की स्थापत्य, चित्रकला, हस्तशिल्प, लोक नृत्य, संगीत</v>
       </c>
       <c r="F83" s="1" t="str">
-        <v>6 UNESCO forts; Painting schools (Mewar, Kishangarh); Kalbelia UNESCO; Rajasthani instruments</v>
+        <v>6 UNESCO forts, Painting schools (Mewar, Kishangarh), Kalbelia UNESCO, Rajasthani instruments</v>
       </c>
       <c r="G83" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5339,7 +5318,7 @@
         <v>भाषा, साहित्य, धार्मिक जीवन, संत, लोक देवता</v>
       </c>
       <c r="F84" s="1" t="str">
-        <v>Dingal-Pingal; PVR; Mirabai-Kabir-Ramdeva-Tejaji; Bishnoi-Jasnathi panth</v>
+        <v>Dingal-Pingal, PVR, Mirabai-Kabir-Ramdeva-Tejaji, Bishnoi-Jasnathi panth</v>
       </c>
       <c r="G84" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5398,7 +5377,7 @@
         <v>राजस्थान का सामाजिक जीवन: मेले, त्यौहार, वेशभूषा</v>
       </c>
       <c r="F85" s="1" t="str">
-        <v>Pushkar-Nagaur-Beneshwar melas; Gangaur-Teej; Rajasthani ornaments; social customs</v>
+        <v>Pushkar-Nagaur-Beneshwar melas, Gangaur-Teej, Rajasthani ornaments, social customs</v>
       </c>
       <c r="G85" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -5457,7 +5436,7 @@
         <v>सिंधु सभ्यता से ब्रिटिश काल: ललित कला, स्थापत्य, साहित्य</v>
       </c>
       <c r="F86" s="1" t="str">
-        <v>Sindhu art; Buddhist stupas; Ajanta-Ellora; Mughal painting; Sanskrit-Pali-Apabhramsha lit</v>
+        <v>Sindhu art, Buddhist stupas, Ajanta-Ellora, Mughal painting, Sanskrit-Pali-Apabhramsha lit</v>
       </c>
       <c r="G86" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5516,7 +5495,7 @@
         <v>प्राचीन एवं मध्यकालीन धार्मिक आंदोलन एवं दर्शन</v>
       </c>
       <c r="F87" s="1" t="str">
-        <v>Bhakti-Sufi; Shankaracharya; Ramanuja; Buddhist-Jain philosophy; Upanishad darsana</v>
+        <v>Bhakti-Sufi, Shankaracharya, Ramanuja, Buddhist-Jain philosophy, Upanishad darsana</v>
       </c>
       <c r="G87" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5575,7 +5554,7 @@
         <v>ब्रिटिश नीतियाँ एवं राजनीतिक-आर्थिक-प्रशासनिक एकीकरण</v>
       </c>
       <c r="F88" s="1" t="str">
-        <v>Permanent Settlement; Subsidiary Alliance; Doctrine of Lapse; 1857; Railway-Telegraph policy</v>
+        <v>Permanent Settlement, Subsidiary Alliance, Doctrine of Lapse, 1857, Railway-Telegraph policy</v>
       </c>
       <c r="G88" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5634,7 +5613,7 @@
         <v>भारतीय राष्ट्रीय आंदोलन: विकास, चरण, प्रमुख योगदानकर्ता</v>
       </c>
       <c r="F89" s="1" t="str">
-        <v>1885-1947 phases; Moderates-Extremists-Gandhian; INA; Partition; Rajasthan's contribution</v>
+        <v>1885-1947 phases, Moderates-Extremists-Gandhian, INA, Partition, Rajasthan's contribution</v>
       </c>
       <c r="G89" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5693,7 +5672,7 @@
         <v>19-20वीं सदी: सामाजिक-धार्मिक सुधार आंदोलन</v>
       </c>
       <c r="F90" s="1" t="str">
-        <v>Brahmo Samaj, Arya Samaj, Ramakrishna Mission, Theosophical; Women reforms</v>
+        <v>Brahmo Samaj, Arya Samaj, Ramakrishna Mission, Theosophical, Women reforms</v>
       </c>
       <c r="G90" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5752,7 +5731,7 @@
         <v>स्वातंत्र्योत्तर राष्ट्र निर्माण (2000 तक)</v>
       </c>
       <c r="F91" s="1" t="str">
-        <v>State reorganisation; Nehruvian institutions; Five Year Plans; Green-White Revolution; 1991 LPG</v>
+        <v>State reorganisation, Nehruvian institutions, Five Year Plans, Green-White Revolution, 1991 LPG</v>
       </c>
       <c r="G91" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -5811,7 +5790,7 @@
         <v>पुनर्जागरण एवं धर्म सुधार</v>
       </c>
       <c r="F92" s="1" t="str">
-        <v>Renaissance causes-impact; Protestant Reformation (Martin Luther); Counter-Reformation</v>
+        <v>Renaissance causes-impact, Protestant Reformation (Martin Luther), Counter-Reformation</v>
       </c>
       <c r="G92" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -5870,7 +5849,7 @@
         <v>अमेरिकी-फ्रांसीसी-औद्योगिक-रूसी क्रांति</v>
       </c>
       <c r="F93" s="1" t="str">
-        <v>1776 American Independence; 1789 French (Liberty-Equality-Fraternity); Industrial Rev. (England); 1917 Russian (Bolshevik)</v>
+        <v>1776 American Independence, 1789 French (Liberty-Equality-Fraternity), Industrial Rev. (England), 1917 Russian (Bolshevik)</v>
       </c>
       <c r="G93" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5929,7 +5908,7 @@
         <v>जर्मनी नाजीवाद, इटली फासीवाद, विश्व युद्ध</v>
       </c>
       <c r="F94" s="1" t="str">
-        <v>Hitler-Mussolini ideology; WWI (1914-18), WWII (1939-45); UN formation; Nuclear bomb</v>
+        <v>Hitler-Mussolini ideology, WWI (1914-18), WWII (1939-45), UN formation, Nuclear bomb</v>
       </c>
       <c r="G94" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -5988,7 +5967,7 @@
         <v>शीत युद्ध</v>
       </c>
       <c r="F95" s="1" t="str">
-        <v>NAM (India's role); USA-USSR rivalry; Cuban crisis; Berlin Wall; Soviet collapse 1991</v>
+        <v>NAM (India's role), USA-USSR rivalry, Cuban crisis, Berlin Wall, Soviet collapse 1991</v>
       </c>
       <c r="G95" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6047,7 +6026,7 @@
         <v>आर्थिक संवृद्धि एवं विकास: HDI, SDG, जलवायु परिवर्तन</v>
       </c>
       <c r="F96" s="1" t="str">
-        <v>GDP-HDI-HPI-MPI; SDG 17; Green GDP; Inclusive Growth; Climate-economy nexus</v>
+        <v>GDP-HDI-HPI-MPI, SDG 17, Green GDP, Inclusive Growth, Climate-economy nexus</v>
       </c>
       <c r="G96" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6106,7 +6085,7 @@
         <v>कृषि: उत्पादकता, भूमि सुधार, वित्त, खाद्य सुरक्षा</v>
       </c>
       <c r="F97" s="1" t="str">
-        <v>Green Revolution; Land ceiling; NABARD; MSP-CACP; PM-KISAN; PMFBY; Food Security Act 2013</v>
+        <v>Green Revolution, Land ceiling, NABARD, MSP-CACP, PM-KISAN, PMFBY, Food Security Act 2013</v>
       </c>
       <c r="G97" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6165,7 +6144,7 @@
         <v>औद्योगिक नीति: LPG; MSME; वैश्वीकरण</v>
       </c>
       <c r="F98" s="1" t="str">
-        <v>1991 reforms; PLI; SEZ; MSME new definition 2020; Make in India; FDI-FPI</v>
+        <v>1991 reforms, PLI, SEZ, MSME new definition 2020, Make in India, FDI-FPI</v>
       </c>
       <c r="G98" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6224,7 +6203,7 @@
         <v>सेवा क्षेत्र एवं आधारभूत संरचना: ऊर्जा, परिवहन</v>
       </c>
       <c r="F99" s="1" t="str">
-        <v>IT sector 54% services GDP; PM Gati Shakti; Bharatmala-Sagarmala-UDAN; DMIC</v>
+        <v>IT sector 54% services GDP, PM Gati Shakti, Bharatmala-Sagarmala-UDAN, DMIC</v>
       </c>
       <c r="G99" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -6283,7 +6262,7 @@
         <v>अंतर्राष्ट्रीय व्यापार, BOP, FDI, विदेशी सहायता</v>
       </c>
       <c r="F100" s="1" t="str">
-        <v>CAD; WTO disputes; India's FDI inflow ranking; BoP crisis 1991; EXIM policy</v>
+        <v>CAD, WTO disputes, India's FDI inflow ranking, BoP crisis 1991, EXIM policy</v>
       </c>
       <c r="G100" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6342,7 +6321,7 @@
         <v>सार्वजनिक वित्त: बजट, राजकोषीय नीति, वित्त आयोग</v>
       </c>
       <c r="F101" s="1" t="str">
-        <v>FRBM; Fiscal-Revenue-Primary Deficit; 15th FC (41%); GST Council; Union Budget 2025-26</v>
+        <v>FRBM, Fiscal-Revenue-Primary Deficit, 15th FC (41%), GST Council, Union Budget 2025-26</v>
       </c>
       <c r="G101" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6401,7 +6380,7 @@
         <v>RBI एवं मौद्रिक प्रबंधन; बैंकिंग सुधार</v>
       </c>
       <c r="F102" s="1" t="str">
-        <v>Repo Rate-CRR-SLR-OMO; MPC; NPA crisis; Bank merger; NBFC regulation; UPI</v>
+        <v>Repo Rate-CRR-SLR-OMO, MPC, NPA crisis, Bank merger, NBFC regulation, UPI</v>
       </c>
       <c r="G102" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6460,7 +6439,7 @@
         <v>सामाजिक क्षेत्र: शिक्षा, स्वास्थ्य, गरीबी, बेरोजगारी</v>
       </c>
       <c r="F103" s="1" t="str">
-        <v>NEP 2020; Ayushman Bharat; MGNREGA; PM-SVANidhi; PMAY; Gig economy</v>
+        <v>NEP 2020, Ayushman Bharat, MGNREGA, PM-SVANidhi, PMAY, Gig economy</v>
       </c>
       <c r="G103" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6519,7 +6498,7 @@
         <v>वैश्विक अर्थव्यवस्था: WTO, World Bank, IMF</v>
       </c>
       <c r="F104" s="1" t="str">
-        <v>WTO: dispute settlement, MFN; IMF: SDR, surveillance; WB: IDA-IBRD; Global recession</v>
+        <v>WTO: dispute settlement, MFN, IMF: SDR, surveillance, WB: IDA-IBRD, Global recession</v>
       </c>
       <c r="G104" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -6578,7 +6557,7 @@
         <v>राजस्थान अर्थव्यवस्था: GSDP, कृषि, उद्योग, योजनाएँ</v>
       </c>
       <c r="F105" s="1" t="str">
-        <v>GSDP ₹14 lakh cr; Solar 1st; Zinc-Marble-Copper; Chiranjeevi; Indira Rasoi; IGNP</v>
+        <v>GSDP ₹14 lakh cr, Solar 1st, Zinc-Marble-Copper, Chiranjeevi, Indira Rasoi, IGNP</v>
       </c>
       <c r="G105" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6637,7 +6616,7 @@
         <v>जाति एवं वर्ग: अवधारणा एवं बदलते आयाम</v>
       </c>
       <c r="F106" s="1" t="str">
-        <v>Caste: structure-function-reservation debate; Rising middle class; Inequality measures; Gini coefficient</v>
+        <v>Caste: structure-function-reservation debate, Rising middle class, Inequality measures, Gini coefficient</v>
       </c>
       <c r="G106" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6696,7 +6675,7 @@
         <v>समसामयिक भारतीय समाज में परिवर्तन</v>
       </c>
       <c r="F107" s="1" t="str">
-        <v>Secularism debate; Urbanisation (Smart Cities); Modernisation vs tradition; Globalisation impact</v>
+        <v>Secularism debate, Urbanisation (Smart Cities), Modernisation vs tradition, Globalisation impact</v>
       </c>
       <c r="G107" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6755,7 +6734,7 @@
         <v>भारतीय सामाजिक व्यवस्था: कर्म, धर्म, पुरुषार्थ, आश्रम</v>
       </c>
       <c r="F108" s="1" t="str">
-        <v>4 Ashrams; 4 Purushartha; Varnashrama; Dharmashastra; Vedanta philosophy</v>
+        <v>4 Ashrams, 4 Purushartha, Varnashrama, Dharmashastra, Vedanta philosophy</v>
       </c>
       <c r="G108" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -6814,7 +6793,7 @@
         <v>परिवार, विवाह, साइबर अपराध, सोशल मीडिया प्रभाव</v>
       </c>
       <c r="F109" s="1" t="str">
-        <v>Joint family breakdown; Marriage forms; Cyber crime (POCSO, IT Act); Social media addiction</v>
+        <v>Joint family breakdown, Marriage forms, Cyber crime (POCSO, IT Act), Social media addiction</v>
       </c>
       <c r="G109" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6873,7 +6852,7 @@
         <v>भारतीय समाज की चुनौतियाँ: दहेज, भ्रष्टाचार, गरीबी, नशा</v>
       </c>
       <c r="F110" s="1" t="str">
-        <v>Dowry Prohibition Act; Corruption index; BPL criteria; NDPS Act; De-addiction</v>
+        <v>Dowry Prohibition Act, Corruption index, BPL criteria, NDPS Act, De-addiction</v>
       </c>
       <c r="G110" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6932,7 +6911,7 @@
         <v>कमजोर वर्गों की समस्याएँ (राजस्थान विशेष)</v>
       </c>
       <c r="F111" s="1" t="str">
-        <v>Women empowerment; Tribal Sub-Plan; SCSP; Rajasthan SC/ST Commission; Dalit welfare</v>
+        <v>Women empowerment, Tribal Sub-Plan, SCSP, Rajasthan SC/ST Commission, Dalit welfare</v>
       </c>
       <c r="G111" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -6991,7 +6970,7 @@
         <v>सामान्य प्रबंध: POSDCORB, MBO, निर्णय प्रक्रिया</v>
       </c>
       <c r="F112" s="1" t="str">
-        <v>POSDCORB (Gulick); MBO (Peter Drucker); Decision Tree; Rational-Bounded Rational model</v>
+        <v>POSDCORB (Gulick), MBO (Peter Drucker), Decision Tree, Rational-Bounded Rational model</v>
       </c>
       <c r="G112" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7050,7 +7029,7 @@
         <v>संगठनात्मक व्यवहार: अभिप्रेरणा, नेतृत्व, समूह गतिशीलता</v>
       </c>
       <c r="F113" s="1" t="str">
-        <v>Maslow, Herzberg (2-factor), McGregor (X-Y); Transformational leadership; Team building</v>
+        <v>Maslow, Herzberg (2-factor), McGregor (X-Y), Transformational leadership, Team building</v>
       </c>
       <c r="G113" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7109,7 +7088,7 @@
         <v>विपणन प्रबंध: 4P→7P; डिजिटल विपणन</v>
       </c>
       <c r="F114" s="1" t="str">
-        <v>Product-Price-Promotion-Place + People-Process-Physical; Digital marketing; E-commerce; CRM</v>
+        <v>Product-Price-Promotion-Place + People-Process-Physical, Digital marketing, E-commerce, CRM</v>
       </c>
       <c r="G114" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -7168,7 +7147,7 @@
         <v>मानव संसाधन प्रबंध: HRP, भर्ती, प्रशिक्षण, PMS</v>
       </c>
       <c r="F115" s="1" t="str">
-        <v>HRP→Recruitment→Selection→T&amp;D→Performance Appraisal; HR Analytics; Gig economy</v>
+        <v>HRP→Recruitment→Selection→T&amp;D→Performance Appraisal, HR Analytics, Gig economy</v>
       </c>
       <c r="G115" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7227,7 +7206,7 @@
         <v>रणनीतिक प्रबंधन: SWOT, Porter's 5 Forces, BCG</v>
       </c>
       <c r="F116" s="1" t="str">
-        <v>SWOT analysis; Porter's 5 Forces; BCG Matrix; Balanced Scorecard; Mission-Vision</v>
+        <v>SWOT analysis, Porter's 5 Forces, BCG Matrix, Balanced Scorecard, Mission-Vision</v>
       </c>
       <c r="G116" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -7286,7 +7265,7 @@
         <v>लेखांकन सिद्धांत: GAAP, मूलभूत अवधारणाएँ</v>
       </c>
       <c r="F117" s="1" t="str">
-        <v>Going Concern, Consistency, Accrual, Materiality; Double Entry; Journal-Ledger-Trial Balance</v>
+        <v>Going Concern, Consistency, Accrual, Materiality, Double Entry, Journal-Ledger-Trial Balance</v>
       </c>
       <c r="G117" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7345,7 +7324,7 @@
         <v>वित्तीय विवरण विश्लेषण; रोकड़ प्रवाह; CSR लेखांकन</v>
       </c>
       <c r="F118" s="1" t="str">
-        <v>P&amp;L, Balance Sheet, Cash Flow; Ratio Analysis (Liquidity, Solvency, Profitability); CSR Accounting</v>
+        <v>P&amp;L, Balance Sheet, Cash Flow, Ratio Analysis (Liquidity, Solvency, Profitability), CSR Accounting</v>
       </c>
       <c r="G118" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7404,7 +7383,7 @@
         <v>GST का आधारभूत ज्ञान</v>
       </c>
       <c r="F119" s="1" t="str">
-        <v>GST slabs (0/5/12/18/28%); CGST-SGST-IGST; Input Tax Credit; e-Invoice; GSTN</v>
+        <v>GST slabs (0/5/12/18/28%), CGST-SGST-IGST, Input Tax Credit, e-Invoice, GSTN</v>
       </c>
       <c r="G119" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7463,7 +7442,7 @@
         <v>अंकेक्षण: CAG, सामाजिक, निष्पादन, दक्षता अंकेक्षण</v>
       </c>
       <c r="F120" s="1" t="str">
-        <v>CAG: Art.148; Performance Audit; Social Audit (MGNREGA); VFM Audit; Government Audit process</v>
+        <v>CAG: Art.148, Performance Audit, Social Audit (MGNREGA), VFM Audit, Government Audit process</v>
       </c>
       <c r="G120" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7522,7 +7501,7 @@
         <v>नीतिशास्त्र एवं मानवीय मूल्य: महापुरुषों से शिक्षा</v>
       </c>
       <c r="F121" s="1" t="str">
-        <v>Gandhi, Lincoln, Mandela, APJ Kalam; Family-Social-Educational institutions' role in ethics</v>
+        <v>Gandhi, Lincoln, Mandela, APJ Kalam, Family-Social-Educational institutions' role in ethics</v>
       </c>
       <c r="G121" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7640,7 +7619,7 @@
         <v>सार्वजनिक एवं निजी जीवन में नीतिशास्त्र; पारदर्शिता</v>
       </c>
       <c r="F123" s="1" t="str">
-        <v>RTI + Whistleblower; Open Government; Integrity-Impartiality-Non-attachment (दार्शनिक आधार)</v>
+        <v>RTI + Whistleblower, Open Government, Integrity-Impartiality-Non-attachment (दार्शनिक आधार)</v>
       </c>
       <c r="G123" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7699,7 +7678,7 @@
         <v>भगवद् गीता का नीतिशास्त्र; गाँधी का नीतिशास्त्र</v>
       </c>
       <c r="F124" s="1" t="str">
-        <v>निष्काम कर्म; Trusteeship; Sarvodaya; Gram Swaraj; Civil Disobedience; Truth-Nonviolence</v>
+        <v>निष्काम कर्म, Trusteeship, Sarvodaya, Gram Swaraj, Civil Disobedience, Truth-Nonviolence</v>
       </c>
       <c r="G124" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7758,7 +7737,7 @@
         <v>भारतीय एवं विश्व नैतिक चिंतक एवं दार्शनिक</v>
       </c>
       <c r="F125" s="1" t="str">
-        <v>Chanakya, Vivekananda, Ambedkar; Aristotle, Socrates, Rawls (Justice), Peter Singer</v>
+        <v>Chanakya, Vivekananda, Ambedkar, Aristotle, Socrates, Rawls (Justice), Peter Singer</v>
       </c>
       <c r="G125" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -7817,7 +7796,7 @@
         <v>प्रशासन में नैतिक द्वंद्व; AI बनाम अंतर्विवेक; नैतिक निर्णय</v>
       </c>
       <c r="F126" s="1" t="str">
-        <v>Conflict of Interest; Whistleblowing; AI Ethics (algorithmic bias); Social Justice; Accountability</v>
+        <v>Conflict of Interest, Whistleblowing, AI Ethics (algorithmic bias), Social Justice, Accountability</v>
       </c>
       <c r="G126" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7876,7 +7855,7 @@
         <v>अ-तथ्यपरक केस अध्ययन (Case Studies)</v>
       </c>
       <c r="F127" s="1" t="str">
-        <v>Scenario-based ethical dilemmas: IAS officer under political pressure; RTI whistleblower; Bribe</v>
+        <v>Scenario-based ethical dilemmas: IAS officer under political pressure, RTI whistleblower, Bribe</v>
       </c>
       <c r="G127" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7935,7 +7914,7 @@
         <v>दैनिक जीवन में रसायन विज्ञान: परमाणु संरचना, धातु-अधातु, अम्ल-क्षार, औषधियाँ, कार्बन, ईंधन, रेडियोधर्मिता</v>
       </c>
       <c r="F128" s="1" t="str">
-        <v>Periodic Table; pH-buffer; Medicines (synthetic-natural); Antioxidants; Carbon allotropes; Octane rating; Radioactive decay; Green Chemistry</v>
+        <v>Periodic Table, pH-buffer, Medicines (synthetic-natural), Antioxidants, Carbon allotropes, Octane rating, Radioactive decay, Green Chemistry</v>
       </c>
       <c r="G128" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -7994,7 +7973,7 @@
         <v>दैनिक जीवन में भौतिकी: गति, प्रकाश, ऊष्मा, विद्युत, चुम्बकत्व, ध्वनि, नाभिकीय विखंडन-संलयन</v>
       </c>
       <c r="F129" s="1" t="str">
-        <v>Laws of Motion; Light (LASER-Fibre Optics); X-Ray-MRI-Ultrasound; Nuclear Reactor; Radiation safety</v>
+        <v>Laws of Motion, Light (LASER-Fibre Optics), X-Ray-MRI-Ultrasound, Nuclear Reactor, Radiation safety</v>
       </c>
       <c r="G129" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8053,7 +8032,7 @@
         <v>जीव विज्ञान: कोशिका, पोषण, मानव शरीर, रोग, जैवप्रौद्योगिकी, GMO</v>
       </c>
       <c r="F130" s="1" t="str">
-        <v>Cell organelles; Digestive-Respiratory-Circulatory systems; Vaccines; Bt crops; CRISPR-Cas9; mRNA vaccine; ELSI of GMO</v>
+        <v>Cell organelles, Digestive-Respiratory-Circulatory systems, Vaccines, Bt crops, CRISPR-Cas9, mRNA vaccine, ELSI of GMO</v>
       </c>
       <c r="G130" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8112,7 +8091,7 @@
         <v>ICT: AI, ML, Big Data, Cloud, IoT, Blockchain, 5G, OTT</v>
       </c>
       <c r="F131" s="1" t="str">
-        <v>AI vs ML vs DL; GPT models; IoT applications; Blockchain = distributed ledger; 5G spectrum; Cybercrime types</v>
+        <v>AI vs ML vs DL, GPT models, IoT applications, Blockchain = distributed ledger, 5G spectrum, Cybercrime types</v>
       </c>
       <c r="G131" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8171,7 +8150,7 @@
         <v>भारतीय वैज्ञानिक संस्थान एवं S&amp;T नीतियाँ; Robotics, Nanotechnology, Quantum Computing</v>
       </c>
       <c r="F132" s="1" t="str">
-        <v>ISRO, DRDO, CSIR, IISc, BARC; Chandrayaan-3; National Quantum Mission 2023; BioE3 Policy 2024; Atmanirbhar Bharat defence</v>
+        <v>ISRO, DRDO, CSIR, IISc, BARC, Chandrayaan-3, National Quantum Mission 2023, BioE3 Policy 2024, Atmanirbhar Bharat defence</v>
       </c>
       <c r="G132" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8230,7 +8209,7 @@
         <v>अंतरिक्ष एवं रक्षा प्रौद्योगिकी: ISRO, उपग्रह, मिसाइल, ड्रोन, रासायनिक-जैविक हथियार</v>
       </c>
       <c r="F133" s="1" t="str">
-        <v>PSLV/GSLV/LVM3; Gaganyaan; OneWeb-GSAT; Agni-V MIRV; BrahMos; Tejas HAL; CWC (Chemical Weapons Convention)</v>
+        <v>PSLV/GSLV/LVM3, Gaganyaan, OneWeb-GSAT, Agni-V MIRV, BrahMos, Tejas HAL, CWC (Chemical Weapons Convention)</v>
       </c>
       <c r="G133" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8289,7 +8268,7 @@
         <v>विश्व: पृथ्वी संरचना, भू-आकृतियाँ, भूकम्प, ज्वालामुखी, जलवायु</v>
       </c>
       <c r="F134" s="1" t="str">
-        <v>Internal structure; Plate Tectonics; Richter-Mercalli; Ring of Fire; Hadley Cell; ITCZ; El Nino</v>
+        <v>Internal structure, Plate Tectonics, Richter-Mercalli, Ring of Fire, Hadley Cell, ITCZ, El Nino</v>
       </c>
       <c r="G134" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8348,7 +8327,7 @@
         <v>पर्यावरणीय मुद्दे (विश्व)</v>
       </c>
       <c r="F135" s="1" t="str">
-        <v>Global Warming; Ozone depletion (Montreal 1987); Acid Rain; Biodiversity loss; COP28</v>
+        <v>Global Warming, Ozone depletion (Montreal 1987), Acid Rain, Biodiversity loss, COP28</v>
       </c>
       <c r="G135" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8407,7 +8386,7 @@
         <v>भारत: भौतिक विभाजन, जलवायु, नदियाँ, संसाधन, जनसंख्या</v>
       </c>
       <c r="F136" s="1" t="str">
-        <v>Himalaya-Plain-Plateau; SW Monsoon; Ganga-Brahmaputra; Coal-Iron ore; Census 2011 data</v>
+        <v>Himalaya-Plain-Plateau, SW Monsoon, Ganga-Brahmaputra, Coal-Iron ore, Census 2011 data</v>
       </c>
       <c r="G136" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8466,7 +8445,7 @@
         <v>राजस्थान: भौतिक विभाग, जलवायु, वनस्पति, खनिज, जनजातियाँ, UNESCO Geopark</v>
       </c>
       <c r="F137" s="1" t="str">
-        <v>4 physical divisions; River drainage; Mineral map; Bhil-Meena tribes; Geopark prospects</v>
+        <v>4 physical divisions, River drainage, Mineral map, Bhil-Meena tribes, Geopark prospects</v>
       </c>
       <c r="G137" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8525,7 +8504,7 @@
         <v>संविधान: Constituent Assembly, FR, DPSP, FD, Basic Structure</v>
       </c>
       <c r="F138" s="1" t="str">
-        <v>Ambedkar role; Preamble (42nd amend.); FR Art.12-35; DPSP 36-51; Kesavananda Bharati</v>
+        <v>Ambedkar role, Preamble (42nd amend.), FR Art.12-35, DPSP 36-51, Kesavananda Bharati</v>
       </c>
       <c r="G138" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8584,7 +8563,7 @@
         <v>संशोधन प्रक्रिया; प्रमुख संवैधानिक परिवर्तन</v>
       </c>
       <c r="F139" s="1" t="str">
-        <v>Art.368; 42nd, 44th, 73rd, 74th, 97th, 101st Amend.; Basic Structure doctrine</v>
+        <v>Art.368, 42nd, 44th, 73rd, 74th, 97th, 101st Amend., Basic Structure doctrine</v>
       </c>
       <c r="G139" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8643,7 +8622,7 @@
         <v>नवीन न्यायिक निर्णय; संवैधानिक नैतिकता</v>
       </c>
       <c r="F140" s="1" t="str">
-        <v>Navtej Singh Johar; Sabarimala; Right to Privacy (Puttaswamy 2017); EWS reservation (2022)</v>
+        <v>Navtej Singh Johar, Sabarimala, Right to Privacy (Puttaswamy 2017), EWS reservation (2022)</v>
       </c>
       <c r="G140" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8702,7 +8681,7 @@
         <v>राष्ट्रपति, PM, मंत्रिपरिषद, संसद</v>
       </c>
       <c r="F141" s="1" t="str">
-        <v>President: discretionary powers + veto; Anti-Defection 10th Schedule; Parliamentary Committees; Zero Hour</v>
+        <v>President: discretionary powers + veto, Anti-Defection 10th Schedule, Parliamentary Committees, Zero Hour</v>
       </c>
       <c r="G141" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8761,7 +8740,7 @@
         <v>संघवाद: उभरती प्रवृत्तियाँ; न्यायपालिका: PIL, ई-कोर्ट</v>
       </c>
       <c r="F142" s="1" t="str">
-        <v>Co-op vs Competitive Federalism; GST Council; NJAC (struck down); PIL origin; Virtual Courts</v>
+        <v>Co-op vs Competitive Federalism, GST Council, NJAC (struck down), PIL origin, Virtual Courts</v>
       </c>
       <c r="G142" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8820,7 +8799,7 @@
         <v>भारतीय राजनीति: दलीय प्रणाली, मतदान व्यवहार, निर्वाचन सुधार</v>
       </c>
       <c r="F143" s="1" t="str">
-        <v>EVM-VVPAT; NOTA; One Nation One Election; Electoral Bonds; Regionalism; Coalition politics</v>
+        <v>EVM-VVPAT, NOTA, One Nation One Election, Electoral Bonds, Regionalism, Coalition politics</v>
       </c>
       <c r="G143" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8879,7 +8858,7 @@
         <v>आंतरिक सुरक्षा: Naxalism, NE Insurgency, J&amp;K; सुरक्षा बल</v>
       </c>
       <c r="F144" s="1" t="str">
-        <v>CRPF, BSF, NSG; NIA; UAPA; Anti-terror laws; LWE Map; Cyber security threats</v>
+        <v>CRPF, BSF, NSG, NIA, UAPA, Anti-terror laws, LWE Map, Cyber security threats</v>
       </c>
       <c r="G144" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8938,7 +8917,7 @@
         <v>राजस्थान राजनीति एवं शासन; e-Governance</v>
       </c>
       <c r="F145" s="1" t="str">
-        <v>2023 elections; Coalition; Raj. PR Act 1994; e-Mitra; Jan Aadhaar; Raj Kaushal Portal</v>
+        <v>2023 elections, Coalition, Raj. PR Act 1994, e-Mitra, Jan Aadhaar, Raj Kaushal Portal</v>
       </c>
       <c r="G145" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -8997,7 +8976,7 @@
         <v>भारत एवं अंतर्राष्ट्रीय मामले: विदेश नीति, QUAD, G20, BRICS</v>
       </c>
       <c r="F146" s="1" t="str">
-        <v>Strategic Autonomy; Neighbourhood First; G20 New Delhi 2023; QUAD; India-Middle East Corridor; DAKSHIN</v>
+        <v>Strategic Autonomy, Neighbourhood First, G20 New Delhi 2023, QUAD, India-Middle East Corridor, DAKSHIN</v>
       </c>
       <c r="G146" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9056,7 +9035,7 @@
         <v>जलवायु कूटनीति; समसामयिक मामले</v>
       </c>
       <c r="F147" s="1" t="str">
-        <v>ISA; Mission LiFE; COP29; Panchamrit; Olympics 2024; Nobel 2024; Bharat Ratna 2024</v>
+        <v>ISA, Mission LiFE, COP29, Panchamrit, Olympics 2024, Nobel 2024, Bharat Ratna 2024</v>
       </c>
       <c r="G147" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9115,7 +9094,7 @@
         <v>लोक प्रशासन: विचारधाराएँ — NPM, सुशासन, नव लोक सेवा</v>
       </c>
       <c r="F148" s="1" t="str">
-        <v>Wilson; Taylor (Scientific Mgmt); NPM (Osborne-Gaebler); Good Governance (UNDP 8 features); NPS</v>
+        <v>Wilson, Taylor (Scientific Mgmt), NPM (Osborne-Gaebler), Good Governance (UNDP 8 features), NPS</v>
       </c>
       <c r="G148" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9174,7 +9153,7 @@
         <v>संगठन के सिद्धांत; प्रशासनिक व्यवहार</v>
       </c>
       <c r="F149" s="1" t="str">
-        <v>Hierarchy; Unity of Command; Span of Control; Delegation; Coordination; Simon's bounded rationality</v>
+        <v>Hierarchy, Unity of Command, Span of Control, Delegation, Coordination, Simon's bounded rationality</v>
       </c>
       <c r="G149" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9233,7 +9212,7 @@
         <v>केंद्रीय प्रशासनिक संस्थाएँ: UPSC, ECI, CAG, FC, Lokpal, NITI Aayog</v>
       </c>
       <c r="F150" s="1" t="str">
-        <v>Constitutional Article for each body; Composition; Functions; Independence mechanism</v>
+        <v>Constitutional Article for each body, Composition, Functions, Independence mechanism</v>
       </c>
       <c r="G150" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9292,7 +9271,7 @@
         <v>कार्मिक प्रशासन: भर्ती, प्रशिक्षण, ACR→APAR, Lateral Entry</v>
       </c>
       <c r="F151" s="1" t="str">
-        <v>UPSC; DPC; All India Services; AIS conduct rules; Lateral entry debate</v>
+        <v>UPSC, DPC, All India Services, AIS conduct rules, Lateral entry debate</v>
       </c>
       <c r="G151" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9351,7 +9330,7 @@
         <v>प्रशासन के मुद्दे: ARC II, सामाजिक अंकेक्षण; नियंत्रण</v>
       </c>
       <c r="F152" s="1" t="str">
-        <v>ARC II recommendations; Social Audit (MGNREGA); CAG; Parliamentary Questions; Ombudsman</v>
+        <v>ARC II recommendations, Social Audit (MGNREGA), CAG, Parliamentary Questions, Ombudsman</v>
       </c>
       <c r="G152" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9410,7 +9389,7 @@
         <v>तुलनात्मक लोक प्रशासन: USA, UK, France, China</v>
       </c>
       <c r="F153" s="1" t="str">
-        <v>Presidential (US) vs Parliamentary (UK); Spoils system; Grands Corps (France); CPC (China)</v>
+        <v>Presidential (US) vs Parliamentary (UK), Spoils system, Grands Corps (France), CPC (China)</v>
       </c>
       <c r="G153" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -9469,7 +9448,7 @@
         <v>राज्य एवं जिला प्रशासन</v>
       </c>
       <c r="F154" s="1" t="str">
-        <v>Governor-CM-Cabinet; State Secretariat; Chief Secretary; District Collector (3 roles); Revenue Administration</v>
+        <v>Governor-CM-Cabinet, State Secretariat, Chief Secretary, District Collector (3 roles), Revenue Administration</v>
       </c>
       <c r="G154" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9528,7 +9507,7 @@
         <v>बुद्धि के प्रकार: IQ, EQ, SQ; Gardner's Multiple Intelligences</v>
       </c>
       <c r="F155" s="1" t="str">
-        <v>Cognitive, Social, Emotional, Cultural, Appreciative, Spiritual; EQ (Goleman) at workplace</v>
+        <v>Cognitive, Social, Emotional, Cultural, Appreciative, Spiritual, EQ (Goleman) at workplace</v>
       </c>
       <c r="G155" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9587,7 +9566,7 @@
         <v>नेतृत्व: सिद्धांत, प्रकार, शैलियाँ</v>
       </c>
       <c r="F156" s="1" t="str">
-        <v>Trait, Behavioral, Situational, Transformational, Servant Leadership; Future leaders' challenges</v>
+        <v>Trait, Behavioral, Situational, Transformational, Servant Leadership, Future leaders' challenges</v>
       </c>
       <c r="G156" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9646,7 +9625,7 @@
         <v>कार्यस्थल संचार; Cyberstalking, Moonlighting</v>
       </c>
       <c r="F157" s="1" t="str">
-        <v>Shannon-Weaver model; Grapevine (informal); Barriers; Electronic destructive communication</v>
+        <v>Shannon-Weaver model, Grapevine (informal), Barriers, Electronic destructive communication</v>
       </c>
       <c r="G157" s="1" t="str">
         <v>⭐ Medium Yield</v>
@@ -9705,7 +9684,7 @@
         <v>बर्नआउट, तनाव; RAISEC Model; लैंगिक मुद्दे</v>
       </c>
       <c r="F158" s="1" t="str">
-        <v>Job Burnout (Maslach); Type A-B personality; RAISEC/Holland's model; Glass Ceiling; POSH Act</v>
+        <v>Job Burnout (Maslach), Type A-B personality, RAISEC/Holland's model, Glass Ceiling, POSH Act</v>
       </c>
       <c r="G158" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9764,7 +9743,7 @@
         <v>RTI Act 2005: Sections 1-20</v>
       </c>
       <c r="F159" s="1" t="str">
-        <v>PIO, APIO; Third party info; Sec.8 exemptions; CIC; Penalty provisions; Suo motu disclosure</v>
+        <v>PIO, APIO, Third party info, Sec.8 exemptions, CIC, Penalty provisions, Suo motu disclosure</v>
       </c>
       <c r="G159" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9823,7 +9802,7 @@
         <v>IT Act 2000: Sec.1,2 (definitions), 65,66,66(B-F),67,67(A-C),71-78</v>
       </c>
       <c r="F160" s="1" t="str">
-        <v>Hacking (66), Identity theft (66C), Cyber terrorism (66F), Obscenity (67); Digital signature; CERT-In</v>
+        <v>Hacking (66), Identity theft (66C), Cyber terrorism (66F), Obscenity (67), Digital signature, CERT-In</v>
       </c>
       <c r="G160" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9882,7 +9861,7 @@
         <v>बौद्धिक सम्पदा अधिकार: Patent, Copyright, Trademark, GI Tag</v>
       </c>
       <c r="F161" s="1" t="str">
-        <v>TRIPS Agreement; WIPO; India IPR Policy 2016; GI Tags of Rajasthan (Sanganer Print, Bikaneri Bhujia)</v>
+        <v>TRIPS Agreement, WIPO, India IPR Policy 2016, GI Tags of Rajasthan (Sanganer Print, Bikaneri Bhujia)</v>
       </c>
       <c r="G161" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -9941,7 +9920,7 @@
         <v>महिला-बाल संरक्षण कानून: DV Act 2005, POSH 2013, POCSO 2012, Maintenance Act 2007</v>
       </c>
       <c r="F162" s="1" t="str">
-        <v>DV Act: Sec.1-29,31 (Protection Officer); POSH: ICC-LCC; POCSO: Special Court; Maintenance: Tribunal</v>
+        <v>DV Act: Sec.1-29, 31 (Protection Officer), POSH: ICC-LCC, POCSO: Special Court, Maintenance: Tribunal</v>
       </c>
       <c r="G162" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10000,7 +9979,7 @@
         <v>राजस्थान भूमि विधियाँ: Tenancy Act 1955, Land Revenue Act 1956</v>
       </c>
       <c r="F163" s="1" t="str">
-        <v>Tenancy: Sec.5 (definitions: Khatedar, Bhoomiswami, Grovdharak); Sec.14-17A, 31-37, 38-54A; Revenue: Sec.3 defs</v>
+        <v>Tenancy: Sec.5 (definitions: Khatedar, Bhoomiswami, Grovdharak), Sec.14-17A, 31-37, 38-54A, Revenue: Sec.3 defs</v>
       </c>
       <c r="G163" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10059,7 +10038,7 @@
         <v>BNS 2023 एवं BNSS 2023 (नए आपराधिक कानून)</v>
       </c>
       <c r="F164" s="1" t="str">
-        <v>BNS replaces IPC; Sec.189-191,194-197,270,294-296; BNSS replaces CrPC; FIR, Arrest, Bail, Zero FIR</v>
+        <v>BNS replaces IPC, Sec.189-191, 194-197, 270, 294-296, BNSS replaces CrPC, FIR, Arrest, Bail, Zero FIR</v>
       </c>
       <c r="G164" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10118,7 +10097,7 @@
         <v>उपसर्ग एवं प्रत्यय (30 अंक भाग)</v>
       </c>
       <c r="F165" s="1" t="str">
-        <v>सु/कु/अ/नि/दुर्; इक/ता/त्व/आई — शब्दों से पृथक करना</v>
+        <v>सु/कु/अ/नि/दुर्, इक/ता/त्व/आई — शब्दों से पृथक करना</v>
       </c>
       <c r="G165" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10236,7 +10215,7 @@
         <v>शब्द शुद्धि एवं वाक्य शुद्धि</v>
       </c>
       <c r="F167" s="1" t="str">
-        <v>Common misspellings (उज्जवल→उज्ज्वल); Gender-Number-Karak errors</v>
+        <v>Common misspellings (उज्जवल→उज्ज्वल), Gender-Number-Karak errors</v>
       </c>
       <c r="G167" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10295,7 +10274,7 @@
         <v>मुहावरे एवं लोकोक्तियाँ</v>
       </c>
       <c r="F168" s="1" t="str">
-        <v>100+ मुहावरे (वाक्य प्रयोग सहित); 50 लोकोक्तियाँ</v>
+        <v>100+ मुहावरे (वाक्य प्रयोग सहित), 50 लोकोक्तियाँ</v>
       </c>
       <c r="G168" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10413,7 +10392,7 @@
         <v>संक्षिप्तीकरण (30 अंक भाग)</v>
       </c>
       <c r="F170" s="1" t="str">
-        <v>Passage (150 words) → 1/3 में; Headline → Main body → Key points → Summary style</v>
+        <v>Passage (150 words) → 1/3 में, Headline → Main body → Key points → Summary style</v>
       </c>
       <c r="G170" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10531,7 +10510,7 @@
         <v>अनुवाद: अंग्रेजी → हिंदी</v>
       </c>
       <c r="F172" s="1" t="str">
-        <v>Admin/Legal/Science passages (~50 words); भावानुवाद (literal नहीं)</v>
+        <v>Admin/Legal/Science passages (~50 words), भावानुवाद (literal नहीं)</v>
       </c>
       <c r="G172" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10590,7 +10569,7 @@
         <v>पत्र-लेखन: कार्यालयी पत्र, Office Order, अर्द्धशासकीय, अनुस्मारक, प्रतिवेदन (30 अंक भाग)</v>
       </c>
       <c r="F173" s="1" t="str">
-        <v>Format: Date-सेवा में-विषय-मुख्य भाग-भवदीय; Office Order vs Memo vs DO Letter format</v>
+        <v>Format: Date-सेवा में-विषय-मुख्य भाग-भवदीय, Office Order vs Memo vs DO Letter format</v>
       </c>
       <c r="G173" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10649,7 +10628,7 @@
         <v>प्रारूप-लेखन: अधिसूचना, निविदा, परिपत्र, प्रेस विज्ञप्ति, ज्ञापन</v>
       </c>
       <c r="F174" s="1" t="str">
-        <v>Gazette Notification: structure; Tender Notice: key elements; Press Release: dateline-headline</v>
+        <v>Gazette Notification: structure, Tender Notice: key elements, Press Release: dateline-headline</v>
       </c>
       <c r="G174" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10708,7 +10687,7 @@
         <v>Grammar &amp; Usage: Preposition, Parts of Speech, Phrasal Verbs, Idioms, One Word Sub, Confused Words (20 marks)</v>
       </c>
       <c r="F175" s="1" t="str">
-        <v>Preposition (in/on/at/by/since/for); Same word as noun+verb+adj; 100 Phrasal Verbs; 200 OWS; 50 Confused pairs</v>
+        <v>Preposition (in/on/at/by/since/for), Same word as noun+verb+adj, 100 Phrasal Verbs, 200 OWS, 50 Confused pairs</v>
       </c>
       <c r="G175" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10767,7 +10746,7 @@
         <v>Comprehension (Unseen ~300 words) + Précis Writing ~100 words + Translation Hindi→English (30 marks)</v>
       </c>
       <c r="F176" s="1" t="str">
-        <v>5 questions on passage; Precis = 1/3 length, own words; 5 formal Hindi sentences → idiomatic English</v>
+        <v>5 questions on passage, Precis = 1/3 length, own words, 5 formal Hindi sentences → idiomatic English</v>
       </c>
       <c r="G176" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10826,7 +10805,7 @@
         <v>Elaboration of theme (~150 words); Official Letter / DO Letter / Memo / Report (~150 words) (20 marks)</v>
       </c>
       <c r="F177" s="1" t="str">
-        <v>Theme essay: Intro-3 body para-Conclusion; 5 letter formats with correct heading-salutation-closing</v>
+        <v>Theme essay: Intro-3 body para-Conclusion, 5 letter formats with correct heading-salutation-closing</v>
       </c>
       <c r="G177" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -10885,7 +10864,7 @@
         <v>भाषा, साहित्य एवं सांस्कृतिक विरासत (40 अंक — 600 शब्द)</v>
       </c>
       <c r="F178" s="1" t="str">
-        <v>Hindi/Rajasthani literature; Cultural diversity; Intangible heritage; Classical languages; Linguistic identity</v>
+        <v>Hindi/Rajasthani literature, Cultural diversity, Intangible heritage, Classical languages, Linguistic identity</v>
       </c>
       <c r="G178" s="1" t="str">
         <v>🔥 High Yield</v>
@@ -11232,10 +11211,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B24"/>
-  <cols>
-    <col min="1" max="1" width="60.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -11376,15 +11351,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G8"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">

</xml_diff>

<commit_message>
Update parseExcel.js to ignore header names and parse strictly by column index
</commit_message>
<xml_diff>
--- a/Update_App_Data/ras_syllabus_data.xlsx
+++ b/Update_App_Data/ras_syllabus_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\Storage  Driver\upsc-cse-master-hub\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92701D40-37A4-4BF8-9145-DA8DCE2D8E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF21777B-A8D2-4370-B290-F1B33B61F762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Syllabus!$A$1:$S$183</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -3604,12 +3604,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:S183"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="55" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="96.75" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="118.125" bestFit="1" customWidth="1"/>
@@ -8283,7 +8282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>458</v>
       </c>
@@ -8342,7 +8341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>469</v>
       </c>
@@ -8401,7 +8400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>474</v>
       </c>
@@ -8460,7 +8459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>479</v>
       </c>
@@ -8519,7 +8518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>484</v>
       </c>
@@ -8578,7 +8577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>489</v>
       </c>
@@ -8637,7 +8636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>494</v>
       </c>
@@ -8696,7 +8695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>502</v>
       </c>
@@ -8755,7 +8754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>507</v>
       </c>
@@ -8814,7 +8813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>512</v>
       </c>
@@ -8873,7 +8872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>517</v>
       </c>
@@ -8932,7 +8931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>522</v>
       </c>
@@ -8991,7 +8990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>526</v>
       </c>
@@ -9050,7 +9049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>534</v>
       </c>
@@ -9109,7 +9108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>539</v>
       </c>
@@ -9168,7 +9167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>544</v>
       </c>
@@ -9227,7 +9226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>549</v>
       </c>
@@ -9286,7 +9285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>557</v>
       </c>
@@ -9345,7 +9344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>562</v>
       </c>
@@ -9404,7 +9403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>567</v>
       </c>
@@ -9463,7 +9462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>572</v>
       </c>
@@ -9522,7 +9521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>577</v>
       </c>
@@ -9581,7 +9580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>582</v>
       </c>
@@ -9640,7 +9639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>587</v>
       </c>
@@ -9699,7 +9698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>592</v>
       </c>
@@ -9758,7 +9757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>598</v>
       </c>
@@ -9817,7 +9816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>604</v>
       </c>
@@ -9876,7 +9875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>612</v>
       </c>
@@ -9935,7 +9934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>617</v>
       </c>
@@ -9994,7 +9993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>622</v>
       </c>
@@ -10053,7 +10052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>627</v>
       </c>
@@ -10112,7 +10111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>632</v>
       </c>
@@ -10171,7 +10170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>637</v>
       </c>
@@ -10230,7 +10229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>645</v>
       </c>
@@ -10289,7 +10288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>650</v>
       </c>
@@ -10348,7 +10347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>655</v>
       </c>
@@ -10407,7 +10406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>660</v>
       </c>
@@ -10466,7 +10465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>665</v>
       </c>
@@ -10525,7 +10524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>673</v>
       </c>
@@ -10584,7 +10583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>678</v>
       </c>
@@ -10643,7 +10642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>683</v>
       </c>
@@ -10702,7 +10701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>688</v>
       </c>
@@ -10761,7 +10760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>699</v>
       </c>
@@ -10820,7 +10819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>703</v>
       </c>
@@ -10879,7 +10878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>708</v>
       </c>
@@ -10938,7 +10937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>713</v>
       </c>
@@ -10997,7 +10996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>718</v>
       </c>
@@ -11056,7 +11055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>723</v>
       </c>
@@ -11115,7 +11114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>728</v>
       </c>
@@ -11174,7 +11173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>736</v>
       </c>
@@ -11233,7 +11232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>741</v>
       </c>
@@ -11292,7 +11291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>746</v>
       </c>
@@ -11351,7 +11350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>751</v>
       </c>
@@ -11410,7 +11409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>756</v>
       </c>
@@ -11469,7 +11468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>761</v>
       </c>
@@ -11528,7 +11527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>768</v>
       </c>
@@ -11587,7 +11586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>773</v>
       </c>
@@ -11646,7 +11645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>778</v>
       </c>
@@ -11705,7 +11704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>783</v>
       </c>
@@ -11764,7 +11763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>792</v>
       </c>
@@ -11823,7 +11822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>797</v>
       </c>
@@ -11882,7 +11881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>802</v>
       </c>
@@ -11941,7 +11940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>807</v>
       </c>
@@ -12000,7 +11999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>812</v>
       </c>
@@ -12059,7 +12058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>817</v>
       </c>
@@ -12118,7 +12117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>822</v>
       </c>
@@ -12177,7 +12176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>827</v>
       </c>
@@ -12236,7 +12235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>832</v>
       </c>
@@ -12295,7 +12294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>837</v>
       </c>
@@ -12354,7 +12353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>844</v>
       </c>
@@ -12413,7 +12412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>849</v>
       </c>
@@ -12472,7 +12471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>854</v>
       </c>
@@ -12531,7 +12530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>859</v>
       </c>
@@ -12590,7 +12589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>864</v>
       </c>
@@ -12649,7 +12648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>869</v>
       </c>
@@ -12708,7 +12707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>874</v>
       </c>
@@ -12767,7 +12766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>881</v>
       </c>
@@ -12826,7 +12825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>886</v>
       </c>
@@ -12885,7 +12884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>891</v>
       </c>
@@ -12944,7 +12943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>896</v>
       </c>
@@ -13003,7 +13002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>903</v>
       </c>
@@ -13062,7 +13061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>908</v>
       </c>
@@ -13121,7 +13120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>913</v>
       </c>
@@ -13180,7 +13179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>918</v>
       </c>
@@ -13239,7 +13238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>923</v>
       </c>
@@ -13298,7 +13297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>928</v>
       </c>
@@ -13357,7 +13356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>938</v>
       </c>
@@ -13416,7 +13415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>942</v>
       </c>
@@ -13475,7 +13474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>947</v>
       </c>
@@ -13534,7 +13533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>952</v>
       </c>
@@ -13593,7 +13592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>956</v>
       </c>
@@ -13652,7 +13651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>962</v>
       </c>
@@ -13711,7 +13710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>966</v>
       </c>
@@ -13770,7 +13769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>971</v>
       </c>
@@ -13829,7 +13828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>977</v>
       </c>
@@ -13888,7 +13887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>982</v>
       </c>
@@ -13947,7 +13946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>990</v>
       </c>
@@ -14006,7 +14005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>996</v>
       </c>
@@ -14065,7 +14064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>1002</v>
       </c>
@@ -14124,7 +14123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>1011</v>
       </c>
@@ -14183,7 +14182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>1015</v>
       </c>
@@ -14242,7 +14241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>1019</v>
       </c>
@@ -14301,7 +14300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>1023</v>
       </c>
@@ -14360,7 +14359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>1027</v>
       </c>
@@ -14420,13 +14419,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S183" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Prelims GS1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:S183" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Upgrade Nav tabs to Pro-level Premium UI and add OCR tab
</commit_message>
<xml_diff>
--- a/Update_App_Data/ras_syllabus_data.xlsx
+++ b/Update_App_Data/ras_syllabus_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\New folder (3)\CSE PREP\Update_App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51F872C-76BE-4EA4-B8C7-03FACA7DBAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40FF3CE9-AAE5-4D07-BD3A-1F17F1477691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Syllabus" sheetId="1" r:id="rId1"/>
@@ -3604,6 +3604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:S183"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3682,7 +3683,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -3741,7 +3742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>35</v>
       </c>
@@ -3800,7 +3801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>43</v>
       </c>
@@ -3859,7 +3860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>51</v>
       </c>
@@ -3918,7 +3919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>55</v>
       </c>
@@ -3977,7 +3978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>61</v>
       </c>
@@ -4036,7 +4037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>67</v>
       </c>
@@ -4095,7 +4096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>71</v>
       </c>
@@ -4154,7 +4155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>75</v>
       </c>
@@ -4213,7 +4214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>79</v>
       </c>
@@ -4272,7 +4273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>83</v>
       </c>
@@ -4331,7 +4332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>87</v>
       </c>
@@ -4390,7 +4391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>94</v>
       </c>
@@ -4449,7 +4450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>100</v>
       </c>
@@ -4508,7 +4509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>105</v>
       </c>
@@ -4567,7 +4568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>110</v>
       </c>
@@ -4626,7 +4627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>114</v>
       </c>
@@ -4685,7 +4686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>118</v>
       </c>
@@ -4744,7 +4745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>125</v>
       </c>
@@ -4803,7 +4804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>131</v>
       </c>
@@ -4862,7 +4863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>136</v>
       </c>
@@ -4921,7 +4922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>141</v>
       </c>
@@ -4980,7 +4981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>147</v>
       </c>
@@ -5039,7 +5040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>152</v>
       </c>
@@ -5098,7 +5099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>158</v>
       </c>
@@ -5157,7 +5158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>164</v>
       </c>
@@ -5216,7 +5217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>169</v>
       </c>
@@ -5275,7 +5276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>174</v>
       </c>
@@ -5334,7 +5335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>179</v>
       </c>
@@ -5393,7 +5394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>185</v>
       </c>
@@ -5452,7 +5453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>192</v>
       </c>
@@ -5511,7 +5512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>197</v>
       </c>
@@ -5570,7 +5571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>203</v>
       </c>
@@ -5629,7 +5630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>208</v>
       </c>
@@ -5688,7 +5689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>214</v>
       </c>
@@ -5747,7 +5748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>221</v>
       </c>
@@ -5806,7 +5807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>226</v>
       </c>
@@ -5865,7 +5866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>231</v>
       </c>
@@ -5924,7 +5925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>236</v>
       </c>
@@ -5983,7 +5984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>241</v>
       </c>
@@ -6042,7 +6043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>247</v>
       </c>
@@ -6101,7 +6102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>254</v>
       </c>
@@ -6160,7 +6161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>260</v>
       </c>
@@ -6219,7 +6220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>265</v>
       </c>
@@ -6278,7 +6279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>271</v>
       </c>
@@ -6337,7 +6338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>278</v>
       </c>
@@ -6396,7 +6397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>284</v>
       </c>
@@ -6455,7 +6456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>290</v>
       </c>
@@ -6514,7 +6515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>295</v>
       </c>
@@ -6573,7 +6574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>301</v>
       </c>
@@ -6632,7 +6633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>308</v>
       </c>
@@ -6691,7 +6692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>314</v>
       </c>
@@ -6750,7 +6751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>320</v>
       </c>
@@ -6809,7 +6810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>324</v>
       </c>
@@ -6868,7 +6869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>330</v>
       </c>
@@ -6927,7 +6928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>336</v>
       </c>
@@ -6986,7 +6987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>342</v>
       </c>
@@ -7045,7 +7046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>348</v>
       </c>
@@ -7104,7 +7105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>354</v>
       </c>
@@ -7163,7 +7164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>360</v>
       </c>
@@ -7222,7 +7223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>366</v>
       </c>
@@ -7281,7 +7282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>373</v>
       </c>
@@ -7340,7 +7341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>377</v>
       </c>
@@ -7399,7 +7400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>382</v>
       </c>
@@ -7458,7 +7459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>387</v>
       </c>
@@ -7517,7 +7518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>393</v>
       </c>
@@ -7576,7 +7577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>397</v>
       </c>
@@ -7635,7 +7636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>402</v>
       </c>
@@ -7694,7 +7695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>408</v>
       </c>
@@ -7753,7 +7754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>413</v>
       </c>
@@ -7812,7 +7813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>417</v>
       </c>
@@ -7871,7 +7872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>421</v>
       </c>
@@ -7930,7 +7931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>426</v>
       </c>
@@ -7989,7 +7990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>431</v>
       </c>
@@ -8048,7 +8049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>438</v>
       </c>
@@ -8107,7 +8108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>443</v>
       </c>
@@ -8166,7 +8167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>447</v>
       </c>
@@ -8225,7 +8226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>452</v>
       </c>
@@ -8284,7 +8285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>457</v>
       </c>
@@ -8343,7 +8344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>468</v>
       </c>
@@ -8402,7 +8403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>473</v>
       </c>
@@ -8461,7 +8462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>478</v>
       </c>
@@ -8520,7 +8521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>483</v>
       </c>
@@ -8579,7 +8580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>488</v>
       </c>
@@ -8638,7 +8639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>493</v>
       </c>
@@ -8697,7 +8698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>501</v>
       </c>
@@ -8756,7 +8757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>506</v>
       </c>
@@ -8815,7 +8816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>511</v>
       </c>
@@ -8874,7 +8875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>516</v>
       </c>
@@ -8933,7 +8934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>521</v>
       </c>
@@ -8992,7 +8993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>525</v>
       </c>
@@ -9051,7 +9052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>533</v>
       </c>
@@ -9110,7 +9111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>538</v>
       </c>
@@ -9169,7 +9170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>543</v>
       </c>
@@ -9228,7 +9229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>548</v>
       </c>
@@ -9287,7 +9288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>556</v>
       </c>
@@ -9346,7 +9347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>561</v>
       </c>
@@ -9405,7 +9406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>566</v>
       </c>
@@ -9464,7 +9465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>571</v>
       </c>
@@ -9523,7 +9524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>576</v>
       </c>
@@ -9582,7 +9583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>581</v>
       </c>
@@ -9641,7 +9642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>586</v>
       </c>
@@ -9700,7 +9701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>591</v>
       </c>
@@ -9759,7 +9760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>597</v>
       </c>
@@ -9818,7 +9819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>603</v>
       </c>
@@ -9877,7 +9878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>611</v>
       </c>
@@ -9936,7 +9937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>616</v>
       </c>
@@ -9995,7 +9996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>621</v>
       </c>
@@ -10054,7 +10055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>626</v>
       </c>
@@ -10113,7 +10114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>631</v>
       </c>
@@ -10172,7 +10173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>636</v>
       </c>
@@ -10231,7 +10232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>644</v>
       </c>
@@ -10290,7 +10291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>649</v>
       </c>
@@ -10349,7 +10350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>654</v>
       </c>
@@ -10408,7 +10409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>659</v>
       </c>
@@ -10467,7 +10468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>664</v>
       </c>
@@ -10526,7 +10527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>672</v>
       </c>
@@ -10585,7 +10586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>677</v>
       </c>
@@ -10644,7 +10645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>682</v>
       </c>
@@ -10703,7 +10704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>687</v>
       </c>
@@ -10762,7 +10763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>698</v>
       </c>
@@ -10821,7 +10822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>702</v>
       </c>
@@ -10880,7 +10881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>707</v>
       </c>
@@ -10939,7 +10940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>712</v>
       </c>
@@ -10998,7 +10999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>717</v>
       </c>
@@ -11057,7 +11058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>722</v>
       </c>
@@ -11116,7 +11117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>727</v>
       </c>
@@ -11175,7 +11176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>735</v>
       </c>
@@ -11234,7 +11235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>740</v>
       </c>
@@ -11293,7 +11294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>745</v>
       </c>
@@ -11352,7 +11353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>750</v>
       </c>
@@ -11411,7 +11412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>755</v>
       </c>
@@ -11470,7 +11471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>760</v>
       </c>
@@ -11529,7 +11530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>767</v>
       </c>
@@ -11588,7 +11589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>772</v>
       </c>
@@ -11647,7 +11648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>777</v>
       </c>
@@ -11706,7 +11707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>782</v>
       </c>
@@ -11765,7 +11766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>791</v>
       </c>
@@ -11824,7 +11825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>796</v>
       </c>
@@ -11883,7 +11884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>801</v>
       </c>
@@ -11942,7 +11943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>806</v>
       </c>
@@ -12001,7 +12002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>811</v>
       </c>
@@ -12060,7 +12061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>816</v>
       </c>
@@ -12119,7 +12120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>821</v>
       </c>
@@ -12178,7 +12179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>826</v>
       </c>
@@ -12237,7 +12238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>831</v>
       </c>
@@ -12296,7 +12297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>836</v>
       </c>
@@ -12355,7 +12356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>843</v>
       </c>
@@ -12414,7 +12415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>848</v>
       </c>
@@ -12473,7 +12474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>853</v>
       </c>
@@ -12532,7 +12533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>858</v>
       </c>
@@ -12591,7 +12592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>863</v>
       </c>
@@ -12650,7 +12651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>868</v>
       </c>
@@ -12709,7 +12710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>873</v>
       </c>
@@ -12768,7 +12769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>880</v>
       </c>
@@ -12827,7 +12828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>885</v>
       </c>
@@ -12886,7 +12887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>890</v>
       </c>
@@ -12945,7 +12946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>895</v>
       </c>
@@ -13004,7 +13005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>902</v>
       </c>
@@ -13063,7 +13064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>907</v>
       </c>
@@ -13122,7 +13123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>912</v>
       </c>
@@ -13181,7 +13182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:19" ht="47.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>917</v>
       </c>
@@ -13240,7 +13241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:19" ht="31.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>922</v>
       </c>
@@ -14421,7 +14422,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S183" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:S183" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="14">
+      <filters>
+        <filter val="सामान्य हिंदी एवं सामान्य अंग्रेजी (200 अंक | वर्णनात्मक)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>